<commit_message>
Berlin 2026 : aligner les finishers sur le classement officiel
BMW Berlin Marathon : 50084 -> 50071
Generali Berlin Half Marathon : 36587 -> 36642

Dans les deux cas le compte vient du classement officiel paginate, source la
plus directe. Ajout des chronos vainqueurs du semi (00:59:11 / 01:05:07), que
le plancher de chrono de marathon rejetait jusqu'ici.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01NDRDdaoD47bJRT7WbM1up5
</commit_message>
<xml_diff>
--- a/Chronos_Vainqueurs.xlsx
+++ b/Chronos_Vainqueurs.xlsx
@@ -10,7 +10,7 @@
     <sheet name="Chronos Vainqueurs" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Chronos Vainqueurs'!$A$1:$E$971</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Chronos Vainqueurs'!$A$1:$E$972</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -475,7 +475,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E971"/>
+  <dimension ref="A1:E972"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="50" customWidth="1" min="1" max="1"/>
@@ -18240,7 +18240,7 @@
     <row r="711">
       <c r="A711" s="4" t="inlineStr">
         <is>
-          <t>Generali Prague Half Marathon</t>
+          <t>Generali Berlin Half Marathon</t>
         </is>
       </c>
       <c r="B711" s="5" t="inlineStr">
@@ -18249,16 +18249,16 @@
         </is>
       </c>
       <c r="C711" s="5" t="n">
-        <v>2023</v>
+        <v>2026</v>
       </c>
       <c r="D711" s="5" t="inlineStr">
         <is>
-          <t>0:59:43</t>
+          <t>0:59:11</t>
         </is>
       </c>
       <c r="E711" s="5" t="inlineStr">
         <is>
-          <t>1:06:00</t>
+          <t>1:05:07</t>
         </is>
       </c>
     </row>
@@ -18274,16 +18274,16 @@
         </is>
       </c>
       <c r="C712" s="7" t="n">
-        <v>2024</v>
+        <v>2023</v>
       </c>
       <c r="D712" s="7" t="inlineStr">
         <is>
-          <t>0:58:24</t>
+          <t>0:59:43</t>
         </is>
       </c>
       <c r="E712" s="7" t="inlineStr">
         <is>
-          <t>1:08:10</t>
+          <t>1:06:00</t>
         </is>
       </c>
     </row>
@@ -18299,23 +18299,23 @@
         </is>
       </c>
       <c r="C713" s="5" t="n">
-        <v>2025</v>
+        <v>2024</v>
       </c>
       <c r="D713" s="5" t="inlineStr">
         <is>
-          <t>0:58:54</t>
+          <t>0:58:24</t>
         </is>
       </c>
       <c r="E713" s="5" t="inlineStr">
         <is>
-          <t>1:05:27</t>
+          <t>1:08:10</t>
         </is>
       </c>
     </row>
     <row r="714">
       <c r="A714" s="6" t="inlineStr">
         <is>
-          <t>GetPro Bath Half</t>
+          <t>Generali Prague Half Marathon</t>
         </is>
       </c>
       <c r="B714" s="7" t="inlineStr">
@@ -18328,12 +18328,12 @@
       </c>
       <c r="D714" s="7" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>0:58:54</t>
         </is>
       </c>
       <c r="E714" s="7" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>1:05:27</t>
         </is>
       </c>
     </row>
@@ -18349,7 +18349,7 @@
         </is>
       </c>
       <c r="C715" s="5" t="n">
-        <v>2026</v>
+        <v>2025</v>
       </c>
       <c r="D715" s="5" t="inlineStr">
         <is>
@@ -18365,7 +18365,7 @@
     <row r="716">
       <c r="A716" s="6" t="inlineStr">
         <is>
-          <t>Göteborgsvarvet</t>
+          <t>GetPro Bath Half</t>
         </is>
       </c>
       <c r="B716" s="7" t="inlineStr">
@@ -18374,16 +18374,16 @@
         </is>
       </c>
       <c r="C716" s="7" t="n">
-        <v>2000</v>
+        <v>2026</v>
       </c>
       <c r="D716" s="7" t="inlineStr">
         <is>
-          <t>1:02:42</t>
+          <t>N/A</t>
         </is>
       </c>
       <c r="E716" s="7" t="inlineStr">
         <is>
-          <t>1:09:28</t>
+          <t>N/A</t>
         </is>
       </c>
     </row>
@@ -18399,16 +18399,16 @@
         </is>
       </c>
       <c r="C717" s="5" t="n">
-        <v>2001</v>
+        <v>2000</v>
       </c>
       <c r="D717" s="5" t="inlineStr">
         <is>
-          <t>1:03:00</t>
+          <t>1:02:42</t>
         </is>
       </c>
       <c r="E717" s="5" t="inlineStr">
         <is>
-          <t>1:11:07</t>
+          <t>1:09:28</t>
         </is>
       </c>
     </row>
@@ -18424,16 +18424,16 @@
         </is>
       </c>
       <c r="C718" s="7" t="n">
-        <v>2002</v>
+        <v>2001</v>
       </c>
       <c r="D718" s="7" t="inlineStr">
         <is>
-          <t>1:03:35</t>
+          <t>1:03:00</t>
         </is>
       </c>
       <c r="E718" s="7" t="inlineStr">
         <is>
-          <t>1:13:03</t>
+          <t>1:11:07</t>
         </is>
       </c>
     </row>
@@ -18449,16 +18449,16 @@
         </is>
       </c>
       <c r="C719" s="5" t="n">
-        <v>2003</v>
+        <v>2002</v>
       </c>
       <c r="D719" s="5" t="inlineStr">
         <is>
-          <t>1:03:43</t>
+          <t>1:03:35</t>
         </is>
       </c>
       <c r="E719" s="5" t="inlineStr">
         <is>
-          <t>1:13:27</t>
+          <t>1:13:03</t>
         </is>
       </c>
     </row>
@@ -18474,16 +18474,16 @@
         </is>
       </c>
       <c r="C720" s="7" t="n">
-        <v>2004</v>
+        <v>2003</v>
       </c>
       <c r="D720" s="7" t="inlineStr">
         <is>
-          <t>1:04:03</t>
+          <t>1:03:43</t>
         </is>
       </c>
       <c r="E720" s="7" t="inlineStr">
         <is>
-          <t>1:18:06</t>
+          <t>1:13:27</t>
         </is>
       </c>
     </row>
@@ -18499,16 +18499,16 @@
         </is>
       </c>
       <c r="C721" s="5" t="n">
-        <v>2005</v>
+        <v>2004</v>
       </c>
       <c r="D721" s="5" t="inlineStr">
         <is>
-          <t>1:03:19</t>
+          <t>1:04:03</t>
         </is>
       </c>
       <c r="E721" s="5" t="inlineStr">
         <is>
-          <t>1:12:34</t>
+          <t>1:18:06</t>
         </is>
       </c>
     </row>
@@ -18524,11 +18524,11 @@
         </is>
       </c>
       <c r="C722" s="7" t="n">
-        <v>2006</v>
+        <v>2005</v>
       </c>
       <c r="D722" s="7" t="inlineStr">
         <is>
-          <t>1:02:14</t>
+          <t>1:03:19</t>
         </is>
       </c>
       <c r="E722" s="7" t="inlineStr">
@@ -18549,16 +18549,16 @@
         </is>
       </c>
       <c r="C723" s="5" t="n">
-        <v>2007</v>
+        <v>2006</v>
       </c>
       <c r="D723" s="5" t="inlineStr">
         <is>
-          <t>1:04:03</t>
+          <t>1:02:14</t>
         </is>
       </c>
       <c r="E723" s="5" t="inlineStr">
         <is>
-          <t>1:12:38</t>
+          <t>1:12:34</t>
         </is>
       </c>
     </row>
@@ -18574,16 +18574,16 @@
         </is>
       </c>
       <c r="C724" s="7" t="n">
-        <v>2008</v>
+        <v>2007</v>
       </c>
       <c r="D724" s="7" t="inlineStr">
         <is>
-          <t>1:01:21</t>
+          <t>1:04:03</t>
         </is>
       </c>
       <c r="E724" s="7" t="inlineStr">
         <is>
-          <t>1:10:19</t>
+          <t>1:12:38</t>
         </is>
       </c>
     </row>
@@ -18599,16 +18599,16 @@
         </is>
       </c>
       <c r="C725" s="5" t="n">
-        <v>2009</v>
+        <v>2008</v>
       </c>
       <c r="D725" s="5" t="inlineStr">
         <is>
-          <t>1:01:55</t>
+          <t>1:01:21</t>
         </is>
       </c>
       <c r="E725" s="5" t="inlineStr">
         <is>
-          <t>1:11:27</t>
+          <t>1:10:19</t>
         </is>
       </c>
     </row>
@@ -18624,16 +18624,16 @@
         </is>
       </c>
       <c r="C726" s="7" t="n">
-        <v>2010</v>
+        <v>2009</v>
       </c>
       <c r="D726" s="7" t="inlineStr">
         <is>
-          <t>1:01:10</t>
+          <t>1:01:55</t>
         </is>
       </c>
       <c r="E726" s="7" t="inlineStr">
         <is>
-          <t>1:11:40</t>
+          <t>1:11:27</t>
         </is>
       </c>
     </row>
@@ -18649,16 +18649,16 @@
         </is>
       </c>
       <c r="C727" s="5" t="n">
-        <v>2011</v>
+        <v>2010</v>
       </c>
       <c r="D727" s="5" t="inlineStr">
         <is>
-          <t>1:00:52</t>
+          <t>1:01:10</t>
         </is>
       </c>
       <c r="E727" s="5" t="inlineStr">
         <is>
-          <t>1:09:04</t>
+          <t>1:11:40</t>
         </is>
       </c>
     </row>
@@ -18674,16 +18674,16 @@
         </is>
       </c>
       <c r="C728" s="7" t="n">
-        <v>2012</v>
+        <v>2011</v>
       </c>
       <c r="D728" s="7" t="inlineStr">
         <is>
-          <t>1:00:25</t>
+          <t>1:00:52</t>
         </is>
       </c>
       <c r="E728" s="7" t="inlineStr">
         <is>
-          <t>1:09:27</t>
+          <t>1:09:04</t>
         </is>
       </c>
     </row>
@@ -18699,16 +18699,16 @@
         </is>
       </c>
       <c r="C729" s="5" t="n">
-        <v>2013</v>
+        <v>2012</v>
       </c>
       <c r="D729" s="5" t="inlineStr">
         <is>
-          <t>1:03:13</t>
+          <t>1:00:25</t>
         </is>
       </c>
       <c r="E729" s="5" t="inlineStr">
         <is>
-          <t>1:11:29</t>
+          <t>1:09:27</t>
         </is>
       </c>
     </row>
@@ -18724,16 +18724,16 @@
         </is>
       </c>
       <c r="C730" s="7" t="n">
-        <v>2014</v>
+        <v>2013</v>
       </c>
       <c r="D730" s="7" t="inlineStr">
         <is>
-          <t>1:00:36</t>
+          <t>1:03:13</t>
         </is>
       </c>
       <c r="E730" s="7" t="inlineStr">
         <is>
-          <t>1:10:12</t>
+          <t>1:11:29</t>
         </is>
       </c>
     </row>
@@ -18749,16 +18749,16 @@
         </is>
       </c>
       <c r="C731" s="5" t="n">
-        <v>2024</v>
+        <v>2014</v>
       </c>
       <c r="D731" s="5" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>1:00:36</t>
         </is>
       </c>
       <c r="E731" s="5" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>1:10:12</t>
         </is>
       </c>
     </row>
@@ -18774,7 +18774,7 @@
         </is>
       </c>
       <c r="C732" s="7" t="n">
-        <v>2025</v>
+        <v>2024</v>
       </c>
       <c r="D732" s="7" t="inlineStr">
         <is>
@@ -18799,23 +18799,23 @@
         </is>
       </c>
       <c r="C733" s="5" t="n">
-        <v>2026</v>
+        <v>2025</v>
       </c>
       <c r="D733" s="5" t="inlineStr">
         <is>
-          <t>1:03:30</t>
+          <t>N/A</t>
         </is>
       </c>
       <c r="E733" s="5" t="inlineStr">
         <is>
-          <t>1:13:03</t>
+          <t>N/A</t>
         </is>
       </c>
     </row>
     <row r="734">
       <c r="A734" s="6" t="inlineStr">
         <is>
-          <t>HOKA Semi de Paris</t>
+          <t>Göteborgsvarvet</t>
         </is>
       </c>
       <c r="B734" s="7" t="inlineStr">
@@ -18824,16 +18824,16 @@
         </is>
       </c>
       <c r="C734" s="7" t="n">
-        <v>2002</v>
+        <v>2026</v>
       </c>
       <c r="D734" s="7" t="inlineStr">
         <is>
-          <t>1:01:33</t>
+          <t>1:03:30</t>
         </is>
       </c>
       <c r="E734" s="7" t="inlineStr">
         <is>
-          <t>1:11:07</t>
+          <t>1:13:03</t>
         </is>
       </c>
     </row>
@@ -18849,16 +18849,16 @@
         </is>
       </c>
       <c r="C735" s="5" t="n">
-        <v>2012</v>
+        <v>2002</v>
       </c>
       <c r="D735" s="5" t="inlineStr">
         <is>
-          <t>0:59:44</t>
+          <t>1:01:33</t>
         </is>
       </c>
       <c r="E735" s="5" t="inlineStr">
         <is>
-          <t>1:07:55</t>
+          <t>1:11:07</t>
         </is>
       </c>
     </row>
@@ -18874,16 +18874,16 @@
         </is>
       </c>
       <c r="C736" s="7" t="n">
-        <v>2014</v>
+        <v>2012</v>
       </c>
       <c r="D736" s="7" t="inlineStr">
         <is>
-          <t>1:00:08</t>
+          <t>0:59:44</t>
         </is>
       </c>
       <c r="E736" s="7" t="inlineStr">
         <is>
-          <t>1:09:23</t>
+          <t>1:07:55</t>
         </is>
       </c>
     </row>
@@ -18899,16 +18899,16 @@
         </is>
       </c>
       <c r="C737" s="5" t="n">
-        <v>2023</v>
+        <v>2014</v>
       </c>
       <c r="D737" s="5" t="inlineStr">
         <is>
-          <t>0:59:38</t>
+          <t>1:00:08</t>
         </is>
       </c>
       <c r="E737" s="5" t="inlineStr">
         <is>
-          <t>1:06:01</t>
+          <t>1:09:23</t>
         </is>
       </c>
     </row>
@@ -18924,16 +18924,16 @@
         </is>
       </c>
       <c r="C738" s="7" t="n">
-        <v>2024</v>
+        <v>2023</v>
       </c>
       <c r="D738" s="7" t="inlineStr">
         <is>
-          <t>1:00:45</t>
+          <t>0:59:38</t>
         </is>
       </c>
       <c r="E738" s="7" t="inlineStr">
         <is>
-          <t>1:06:58</t>
+          <t>1:06:01</t>
         </is>
       </c>
     </row>
@@ -18949,16 +18949,16 @@
         </is>
       </c>
       <c r="C739" s="5" t="n">
-        <v>2025</v>
+        <v>2024</v>
       </c>
       <c r="D739" s="5" t="inlineStr">
         <is>
-          <t>1:00:16</t>
+          <t>1:00:45</t>
         </is>
       </c>
       <c r="E739" s="5" t="inlineStr">
         <is>
-          <t>1:07:14</t>
+          <t>1:06:58</t>
         </is>
       </c>
     </row>
@@ -18974,23 +18974,23 @@
         </is>
       </c>
       <c r="C740" s="7" t="n">
-        <v>2026</v>
+        <v>2025</v>
       </c>
       <c r="D740" s="7" t="inlineStr">
         <is>
-          <t>1:00:11</t>
+          <t>1:00:16</t>
         </is>
       </c>
       <c r="E740" s="7" t="inlineStr">
         <is>
-          <t>1:05:12</t>
+          <t>1:07:14</t>
         </is>
       </c>
     </row>
     <row r="741">
       <c r="A741" s="4" t="inlineStr">
         <is>
-          <t>Hackney Half Marathon</t>
+          <t>HOKA Semi de Paris</t>
         </is>
       </c>
       <c r="B741" s="5" t="inlineStr">
@@ -19003,19 +19003,19 @@
       </c>
       <c r="D741" s="5" t="inlineStr">
         <is>
-          <t>1:06:34</t>
+          <t>1:00:11</t>
         </is>
       </c>
       <c r="E741" s="5" t="inlineStr">
         <is>
-          <t>1:14:54</t>
+          <t>1:05:12</t>
         </is>
       </c>
     </row>
     <row r="742">
       <c r="A742" s="6" t="inlineStr">
         <is>
-          <t>Half Marathon Munchen by Brooks</t>
+          <t>Hackney Half Marathon</t>
         </is>
       </c>
       <c r="B742" s="7" t="inlineStr">
@@ -19024,23 +19024,23 @@
         </is>
       </c>
       <c r="C742" s="7" t="n">
-        <v>2025</v>
+        <v>2026</v>
       </c>
       <c r="D742" s="7" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>1:06:34</t>
         </is>
       </c>
       <c r="E742" s="7" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>1:14:54</t>
         </is>
       </c>
     </row>
     <row r="743">
       <c r="A743" s="4" t="inlineStr">
         <is>
-          <t>Hoka Runaway Sydney Half Marathon</t>
+          <t>Half Marathon Munchen by Brooks</t>
         </is>
       </c>
       <c r="B743" s="5" t="inlineStr">
@@ -19065,7 +19065,7 @@
     <row r="744">
       <c r="A744" s="6" t="inlineStr">
         <is>
-          <t>Hyundai Meia Maratona</t>
+          <t>Hoka Runaway Sydney Half Marathon</t>
         </is>
       </c>
       <c r="B744" s="7" t="inlineStr">
@@ -19074,7 +19074,7 @@
         </is>
       </c>
       <c r="C744" s="7" t="n">
-        <v>2023</v>
+        <v>2025</v>
       </c>
       <c r="D744" s="7" t="inlineStr">
         <is>
@@ -19099,7 +19099,7 @@
         </is>
       </c>
       <c r="C745" s="5" t="n">
-        <v>2024</v>
+        <v>2023</v>
       </c>
       <c r="D745" s="5" t="inlineStr">
         <is>
@@ -19124,7 +19124,7 @@
         </is>
       </c>
       <c r="C746" s="7" t="n">
-        <v>2025</v>
+        <v>2024</v>
       </c>
       <c r="D746" s="7" t="inlineStr">
         <is>
@@ -19140,7 +19140,7 @@
     <row r="747">
       <c r="A747" s="4" t="inlineStr">
         <is>
-          <t>IU Health 500 Festival Mini-Marathon</t>
+          <t>Hyundai Meia Maratona</t>
         </is>
       </c>
       <c r="B747" s="5" t="inlineStr">
@@ -19174,23 +19174,23 @@
         </is>
       </c>
       <c r="C748" s="7" t="n">
-        <v>2026</v>
+        <v>2025</v>
       </c>
       <c r="D748" s="7" t="inlineStr">
         <is>
-          <t>1:02:27</t>
+          <t>N/A</t>
         </is>
       </c>
       <c r="E748" s="7" t="inlineStr">
         <is>
-          <t>1:10:07</t>
+          <t>N/A</t>
         </is>
       </c>
     </row>
     <row r="749">
       <c r="A749" s="4" t="inlineStr">
         <is>
-          <t>Kagawa Marugame International Half Marathon</t>
+          <t>IU Health 500 Festival Mini-Marathon</t>
         </is>
       </c>
       <c r="B749" s="5" t="inlineStr">
@@ -19203,19 +19203,19 @@
       </c>
       <c r="D749" s="5" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>1:02:27</t>
         </is>
       </c>
       <c r="E749" s="5" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>1:10:07</t>
         </is>
       </c>
     </row>
     <row r="750">
       <c r="A750" s="6" t="inlineStr">
         <is>
-          <t>Life Time Chicago Half Marathon &amp; 5K</t>
+          <t>Kagawa Marugame International Half Marathon</t>
         </is>
       </c>
       <c r="B750" s="7" t="inlineStr">
@@ -19224,7 +19224,7 @@
         </is>
       </c>
       <c r="C750" s="7" t="n">
-        <v>2024</v>
+        <v>2026</v>
       </c>
       <c r="D750" s="7" t="inlineStr">
         <is>
@@ -19249,7 +19249,7 @@
         </is>
       </c>
       <c r="C751" s="5" t="n">
-        <v>2025</v>
+        <v>2024</v>
       </c>
       <c r="D751" s="5" t="inlineStr">
         <is>
@@ -19265,7 +19265,7 @@
     <row r="752">
       <c r="A752" s="6" t="inlineStr">
         <is>
-          <t>London Landmarks Half Marathon</t>
+          <t>Life Time Chicago Half Marathon &amp; 5K</t>
         </is>
       </c>
       <c r="B752" s="7" t="inlineStr">
@@ -19274,7 +19274,7 @@
         </is>
       </c>
       <c r="C752" s="7" t="n">
-        <v>2024</v>
+        <v>2025</v>
       </c>
       <c r="D752" s="7" t="inlineStr">
         <is>
@@ -19299,7 +19299,7 @@
         </is>
       </c>
       <c r="C753" s="5" t="n">
-        <v>2025</v>
+        <v>2024</v>
       </c>
       <c r="D753" s="5" t="inlineStr">
         <is>
@@ -19315,7 +19315,7 @@
     <row r="754">
       <c r="A754" s="6" t="inlineStr">
         <is>
-          <t>Manchester Half Marathon</t>
+          <t>London Landmarks Half Marathon</t>
         </is>
       </c>
       <c r="B754" s="7" t="inlineStr">
@@ -19340,7 +19340,7 @@
     <row r="755">
       <c r="A755" s="4" t="inlineStr">
         <is>
-          <t>Maratona Do Rio</t>
+          <t>Manchester Half Marathon</t>
         </is>
       </c>
       <c r="B755" s="5" t="inlineStr">
@@ -19349,23 +19349,23 @@
         </is>
       </c>
       <c r="C755" s="5" t="n">
-        <v>2026</v>
+        <v>2025</v>
       </c>
       <c r="D755" s="5" t="inlineStr">
         <is>
-          <t>1:01:53</t>
+          <t>N/A</t>
         </is>
       </c>
       <c r="E755" s="5" t="inlineStr">
         <is>
-          <t>1:11:11</t>
+          <t>N/A</t>
         </is>
       </c>
     </row>
     <row r="756">
       <c r="A756" s="6" t="inlineStr">
         <is>
-          <t>Media Maraton de Bogota</t>
+          <t>Maratona Do Rio</t>
         </is>
       </c>
       <c r="B756" s="7" t="inlineStr">
@@ -19374,16 +19374,16 @@
         </is>
       </c>
       <c r="C756" s="7" t="n">
-        <v>2025</v>
+        <v>2026</v>
       </c>
       <c r="D756" s="7" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>1:01:53</t>
         </is>
       </c>
       <c r="E756" s="7" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>1:11:11</t>
         </is>
       </c>
     </row>
@@ -19399,23 +19399,23 @@
         </is>
       </c>
       <c r="C757" s="5" t="n">
-        <v>2026</v>
+        <v>2025</v>
       </c>
       <c r="D757" s="5" t="inlineStr">
         <is>
-          <t>1:01:59</t>
+          <t>N/A</t>
         </is>
       </c>
       <c r="E757" s="5" t="inlineStr">
         <is>
-          <t>1:12:27</t>
+          <t>N/A</t>
         </is>
       </c>
     </row>
     <row r="758">
       <c r="A758" s="6" t="inlineStr">
         <is>
-          <t>Medio Maration Ciudad de Mexico</t>
+          <t>Media Maraton de Bogota</t>
         </is>
       </c>
       <c r="B758" s="7" t="inlineStr">
@@ -19428,19 +19428,19 @@
       </c>
       <c r="D758" s="7" t="inlineStr">
         <is>
-          <t>1:04:36</t>
+          <t>1:01:59</t>
         </is>
       </c>
       <c r="E758" s="7" t="inlineStr">
         <is>
-          <t>1:12:19</t>
+          <t>1:12:27</t>
         </is>
       </c>
     </row>
     <row r="759">
       <c r="A759" s="4" t="inlineStr">
         <is>
-          <t>Medio Maraton de Buenos Aires</t>
+          <t>Medio Maration Ciudad de Mexico</t>
         </is>
       </c>
       <c r="B759" s="5" t="inlineStr">
@@ -19453,19 +19453,19 @@
       </c>
       <c r="D759" s="5" t="inlineStr">
         <is>
-          <t>0:56:50</t>
+          <t>1:04:36</t>
         </is>
       </c>
       <c r="E759" s="5" t="inlineStr">
         <is>
-          <t>1:03:56</t>
+          <t>1:12:19</t>
         </is>
       </c>
     </row>
     <row r="760">
       <c r="A760" s="6" t="inlineStr">
         <is>
-          <t>Medio Maraton de Sevilla</t>
+          <t>Medio Maraton de Buenos Aires</t>
         </is>
       </c>
       <c r="B760" s="7" t="inlineStr">
@@ -19474,16 +19474,16 @@
         </is>
       </c>
       <c r="C760" s="7" t="n">
-        <v>2024</v>
+        <v>2026</v>
       </c>
       <c r="D760" s="7" t="inlineStr">
         <is>
-          <t>0:59:21</t>
+          <t>0:56:50</t>
         </is>
       </c>
       <c r="E760" s="7" t="inlineStr">
         <is>
-          <t>1:07:59</t>
+          <t>1:03:56</t>
         </is>
       </c>
     </row>
@@ -19499,16 +19499,16 @@
         </is>
       </c>
       <c r="C761" s="5" t="n">
-        <v>2025</v>
+        <v>2024</v>
       </c>
       <c r="D761" s="5" t="inlineStr">
         <is>
-          <t>0:59:33</t>
+          <t>0:59:21</t>
         </is>
       </c>
       <c r="E761" s="5" t="inlineStr">
         <is>
-          <t>1:07:18</t>
+          <t>1:07:59</t>
         </is>
       </c>
     </row>
@@ -19524,23 +19524,23 @@
         </is>
       </c>
       <c r="C762" s="7" t="n">
-        <v>2026</v>
+        <v>2025</v>
       </c>
       <c r="D762" s="7" t="inlineStr">
         <is>
-          <t>1:00:24</t>
+          <t>0:59:33</t>
         </is>
       </c>
       <c r="E762" s="7" t="inlineStr">
         <is>
-          <t>1:06:33</t>
+          <t>1:07:18</t>
         </is>
       </c>
     </row>
     <row r="763">
       <c r="A763" s="4" t="inlineStr">
         <is>
-          <t>Mitja Marato Barcelona by Brooks</t>
+          <t>Medio Maraton de Sevilla</t>
         </is>
       </c>
       <c r="B763" s="5" t="inlineStr">
@@ -19549,16 +19549,16 @@
         </is>
       </c>
       <c r="C763" s="5" t="n">
-        <v>2005</v>
+        <v>2026</v>
       </c>
       <c r="D763" s="5" t="inlineStr">
         <is>
-          <t>1:03:29</t>
+          <t>1:00:24</t>
         </is>
       </c>
       <c r="E763" s="5" t="inlineStr">
         <is>
-          <t>1:09:34</t>
+          <t>1:06:33</t>
         </is>
       </c>
     </row>
@@ -19574,16 +19574,16 @@
         </is>
       </c>
       <c r="C764" s="7" t="n">
-        <v>2006</v>
+        <v>2005</v>
       </c>
       <c r="D764" s="7" t="inlineStr">
         <is>
-          <t>1:02:25</t>
+          <t>1:03:29</t>
         </is>
       </c>
       <c r="E764" s="7" t="inlineStr">
         <is>
-          <t>1:09:26</t>
+          <t>1:09:34</t>
         </is>
       </c>
     </row>
@@ -19599,16 +19599,16 @@
         </is>
       </c>
       <c r="C765" s="5" t="n">
-        <v>2007</v>
+        <v>2006</v>
       </c>
       <c r="D765" s="5" t="inlineStr">
         <is>
-          <t>1:03:02</t>
+          <t>1:02:25</t>
         </is>
       </c>
       <c r="E765" s="5" t="inlineStr">
         <is>
-          <t>1:09:05</t>
+          <t>1:09:26</t>
         </is>
       </c>
     </row>
@@ -19624,16 +19624,16 @@
         </is>
       </c>
       <c r="C766" s="7" t="n">
-        <v>2008</v>
+        <v>2007</v>
       </c>
       <c r="D766" s="7" t="inlineStr">
         <is>
-          <t>1:02:39</t>
+          <t>1:03:02</t>
         </is>
       </c>
       <c r="E766" s="7" t="inlineStr">
         <is>
-          <t>1:09:15</t>
+          <t>1:09:05</t>
         </is>
       </c>
     </row>
@@ -19649,16 +19649,16 @@
         </is>
       </c>
       <c r="C767" s="5" t="n">
-        <v>2009</v>
+        <v>2008</v>
       </c>
       <c r="D767" s="5" t="inlineStr">
         <is>
-          <t>1:01:45</t>
+          <t>1:02:39</t>
         </is>
       </c>
       <c r="E767" s="5" t="inlineStr">
         <is>
-          <t>1:09:34</t>
+          <t>1:09:15</t>
         </is>
       </c>
     </row>
@@ -19674,16 +19674,16 @@
         </is>
       </c>
       <c r="C768" s="7" t="n">
-        <v>2010</v>
+        <v>2009</v>
       </c>
       <c r="D768" s="7" t="inlineStr">
         <is>
-          <t>1:03:00</t>
+          <t>1:01:45</t>
         </is>
       </c>
       <c r="E768" s="7" t="inlineStr">
         <is>
-          <t>1:08:52</t>
+          <t>1:09:34</t>
         </is>
       </c>
     </row>
@@ -19699,16 +19699,16 @@
         </is>
       </c>
       <c r="C769" s="5" t="n">
-        <v>2011</v>
+        <v>2010</v>
       </c>
       <c r="D769" s="5" t="inlineStr">
         <is>
-          <t>1:03:06</t>
+          <t>1:03:00</t>
         </is>
       </c>
       <c r="E769" s="5" t="inlineStr">
         <is>
-          <t>1:08:13</t>
+          <t>1:08:52</t>
         </is>
       </c>
     </row>
@@ -19724,16 +19724,16 @@
         </is>
       </c>
       <c r="C770" s="7" t="n">
-        <v>2012</v>
+        <v>2011</v>
       </c>
       <c r="D770" s="7" t="inlineStr">
         <is>
-          <t>1:02:54</t>
+          <t>1:03:06</t>
         </is>
       </c>
       <c r="E770" s="7" t="inlineStr">
         <is>
-          <t>1:10:51</t>
+          <t>1:08:13</t>
         </is>
       </c>
     </row>
@@ -19749,16 +19749,16 @@
         </is>
       </c>
       <c r="C771" s="5" t="n">
-        <v>2013</v>
+        <v>2012</v>
       </c>
       <c r="D771" s="5" t="inlineStr">
         <is>
-          <t>1:01:44</t>
+          <t>1:02:54</t>
         </is>
       </c>
       <c r="E771" s="5" t="inlineStr">
         <is>
-          <t>1:08:28</t>
+          <t>1:10:51</t>
         </is>
       </c>
     </row>
@@ -19774,16 +19774,16 @@
         </is>
       </c>
       <c r="C772" s="7" t="n">
-        <v>2014</v>
+        <v>2013</v>
       </c>
       <c r="D772" s="7" t="inlineStr">
         <is>
-          <t>1:02:55</t>
+          <t>1:01:44</t>
         </is>
       </c>
       <c r="E772" s="7" t="inlineStr">
         <is>
-          <t>1:08:35</t>
+          <t>1:08:28</t>
         </is>
       </c>
     </row>
@@ -19799,16 +19799,16 @@
         </is>
       </c>
       <c r="C773" s="5" t="n">
-        <v>2023</v>
+        <v>2014</v>
       </c>
       <c r="D773" s="5" t="inlineStr">
         <is>
-          <t>0:58:53</t>
+          <t>1:02:55</t>
         </is>
       </c>
       <c r="E773" s="5" t="inlineStr">
         <is>
-          <t>1:04:37</t>
+          <t>1:08:35</t>
         </is>
       </c>
     </row>
@@ -19824,16 +19824,16 @@
         </is>
       </c>
       <c r="C774" s="7" t="n">
-        <v>2024</v>
+        <v>2023</v>
       </c>
       <c r="D774" s="7" t="inlineStr">
         <is>
-          <t>0:59:21</t>
+          <t>0:58:53</t>
         </is>
       </c>
       <c r="E774" s="7" t="inlineStr">
         <is>
-          <t>1:04:28</t>
+          <t>1:04:37</t>
         </is>
       </c>
     </row>
@@ -19849,16 +19849,16 @@
         </is>
       </c>
       <c r="C775" s="5" t="n">
-        <v>2025</v>
+        <v>2024</v>
       </c>
       <c r="D775" s="5" t="inlineStr">
         <is>
-          <t>0:56:42</t>
+          <t>0:59:21</t>
         </is>
       </c>
       <c r="E775" s="5" t="inlineStr">
         <is>
-          <t>1:04:11</t>
+          <t>1:04:28</t>
         </is>
       </c>
     </row>
@@ -19874,23 +19874,23 @@
         </is>
       </c>
       <c r="C776" s="7" t="n">
-        <v>2026</v>
+        <v>2025</v>
       </c>
       <c r="D776" s="7" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>0:56:42</t>
         </is>
       </c>
       <c r="E776" s="7" t="inlineStr">
         <is>
-          <t>1:04:00</t>
+          <t>1:04:11</t>
         </is>
       </c>
     </row>
     <row r="777">
       <c r="A777" s="4" t="inlineStr">
         <is>
-          <t>Movistar Madrid Medio Maraton</t>
+          <t>Mitja Marato Barcelona by Brooks</t>
         </is>
       </c>
       <c r="B777" s="5" t="inlineStr">
@@ -19899,7 +19899,7 @@
         </is>
       </c>
       <c r="C777" s="5" t="n">
-        <v>2025</v>
+        <v>2026</v>
       </c>
       <c r="D777" s="5" t="inlineStr">
         <is>
@@ -19908,14 +19908,14 @@
       </c>
       <c r="E777" s="5" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>1:04:00</t>
         </is>
       </c>
     </row>
     <row r="778">
       <c r="A778" s="6" t="inlineStr">
         <is>
-          <t>NN CPC Loop Den Haag - Half Marathon</t>
+          <t>Movistar Madrid Medio Maraton</t>
         </is>
       </c>
       <c r="B778" s="7" t="inlineStr">
@@ -19953,12 +19953,12 @@
       </c>
       <c r="D779" s="5" t="inlineStr">
         <is>
-          <t>0:59:36</t>
+          <t>N/A</t>
         </is>
       </c>
       <c r="E779" s="5" t="inlineStr">
         <is>
-          <t>1:08:16</t>
+          <t>N/A</t>
         </is>
       </c>
     </row>
@@ -19974,16 +19974,16 @@
         </is>
       </c>
       <c r="C780" s="7" t="n">
-        <v>2026</v>
+        <v>2025</v>
       </c>
       <c r="D780" s="7" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>0:59:36</t>
         </is>
       </c>
       <c r="E780" s="7" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>1:08:16</t>
         </is>
       </c>
     </row>
@@ -20003,19 +20003,19 @@
       </c>
       <c r="D781" s="5" t="inlineStr">
         <is>
-          <t>0:59:48</t>
+          <t>N/A</t>
         </is>
       </c>
       <c r="E781" s="5" t="inlineStr">
         <is>
-          <t>1:07:34</t>
+          <t>N/A</t>
         </is>
       </c>
     </row>
     <row r="782">
       <c r="A782" s="6" t="inlineStr">
         <is>
-          <t>NYCRUNS Brooklyn Experience Half Marathon</t>
+          <t>NN CPC Loop Den Haag - Half Marathon</t>
         </is>
       </c>
       <c r="B782" s="7" t="inlineStr">
@@ -20024,23 +20024,23 @@
         </is>
       </c>
       <c r="C782" s="7" t="n">
-        <v>2025</v>
+        <v>2026</v>
       </c>
       <c r="D782" s="7" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>0:59:48</t>
         </is>
       </c>
       <c r="E782" s="7" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>1:07:34</t>
         </is>
       </c>
     </row>
     <row r="783">
       <c r="A783" s="4" t="inlineStr">
         <is>
-          <t>NYRR RBC Brooklyn Half</t>
+          <t>NYCRUNS Brooklyn Experience Half Marathon</t>
         </is>
       </c>
       <c r="B783" s="5" t="inlineStr">
@@ -20049,16 +20049,16 @@
         </is>
       </c>
       <c r="C783" s="5" t="n">
-        <v>2022</v>
+        <v>2025</v>
       </c>
       <c r="D783" s="5" t="inlineStr">
         <is>
-          <t>1:03:58</t>
+          <t>N/A</t>
         </is>
       </c>
       <c r="E783" s="5" t="inlineStr">
         <is>
-          <t>1:12:54</t>
+          <t>N/A</t>
         </is>
       </c>
     </row>
@@ -20074,16 +20074,16 @@
         </is>
       </c>
       <c r="C784" s="7" t="n">
-        <v>2023</v>
+        <v>2022</v>
       </c>
       <c r="D784" s="7" t="inlineStr">
         <is>
-          <t>1:03:05</t>
+          <t>1:03:58</t>
         </is>
       </c>
       <c r="E784" s="7" t="inlineStr">
         <is>
-          <t>1:11:38</t>
+          <t>1:12:54</t>
         </is>
       </c>
     </row>
@@ -20099,16 +20099,16 @@
         </is>
       </c>
       <c r="C785" s="5" t="n">
-        <v>2024</v>
+        <v>2023</v>
       </c>
       <c r="D785" s="5" t="inlineStr">
         <is>
-          <t>1:04:08</t>
+          <t>1:03:05</t>
         </is>
       </c>
       <c r="E785" s="5" t="inlineStr">
         <is>
-          <t>1:12:41</t>
+          <t>1:11:38</t>
         </is>
       </c>
     </row>
@@ -20124,16 +20124,16 @@
         </is>
       </c>
       <c r="C786" s="7" t="n">
-        <v>2025</v>
+        <v>2024</v>
       </c>
       <c r="D786" s="7" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>1:04:08</t>
         </is>
       </c>
       <c r="E786" s="7" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>1:12:41</t>
         </is>
       </c>
     </row>
@@ -20149,23 +20149,23 @@
         </is>
       </c>
       <c r="C787" s="5" t="n">
-        <v>2026</v>
+        <v>2025</v>
       </c>
       <c r="D787" s="5" t="inlineStr">
         <is>
-          <t>1:04:32</t>
+          <t>N/A</t>
         </is>
       </c>
       <c r="E787" s="5" t="inlineStr">
         <is>
-          <t>1:13:11</t>
+          <t>N/A</t>
         </is>
       </c>
     </row>
     <row r="788">
       <c r="A788" s="6" t="inlineStr">
         <is>
-          <t>Nike Melbourne Marathon Festival</t>
+          <t>NYRR RBC Brooklyn Half</t>
         </is>
       </c>
       <c r="B788" s="7" t="inlineStr">
@@ -20174,23 +20174,23 @@
         </is>
       </c>
       <c r="C788" s="7" t="n">
-        <v>2025</v>
+        <v>2026</v>
       </c>
       <c r="D788" s="7" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>1:04:32</t>
         </is>
       </c>
       <c r="E788" s="7" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>1:13:11</t>
         </is>
       </c>
     </row>
     <row r="789">
       <c r="A789" s="4" t="inlineStr">
         <is>
-          <t>Riyadh Marathon (Half)</t>
+          <t>Nike Melbourne Marathon Festival</t>
         </is>
       </c>
       <c r="B789" s="5" t="inlineStr">
@@ -20199,7 +20199,7 @@
         </is>
       </c>
       <c r="C789" s="5" t="n">
-        <v>2023</v>
+        <v>2025</v>
       </c>
       <c r="D789" s="5" t="inlineStr">
         <is>
@@ -20224,7 +20224,7 @@
         </is>
       </c>
       <c r="C790" s="7" t="n">
-        <v>2024</v>
+        <v>2023</v>
       </c>
       <c r="D790" s="7" t="inlineStr">
         <is>
@@ -20249,7 +20249,7 @@
         </is>
       </c>
       <c r="C791" s="5" t="n">
-        <v>2025</v>
+        <v>2024</v>
       </c>
       <c r="D791" s="5" t="inlineStr">
         <is>
@@ -20274,7 +20274,7 @@
         </is>
       </c>
       <c r="C792" s="7" t="n">
-        <v>2026</v>
+        <v>2025</v>
       </c>
       <c r="D792" s="7" t="inlineStr">
         <is>
@@ -20290,7 +20290,7 @@
     <row r="793">
       <c r="A793" s="4" t="inlineStr">
         <is>
-          <t>Rock 'n' Roll Running Series Las Vegas</t>
+          <t>Riyadh Marathon (Half)</t>
         </is>
       </c>
       <c r="B793" s="5" t="inlineStr">
@@ -20299,7 +20299,7 @@
         </is>
       </c>
       <c r="C793" s="5" t="n">
-        <v>2023</v>
+        <v>2026</v>
       </c>
       <c r="D793" s="5" t="inlineStr">
         <is>
@@ -20324,7 +20324,7 @@
         </is>
       </c>
       <c r="C794" s="7" t="n">
-        <v>2024</v>
+        <v>2023</v>
       </c>
       <c r="D794" s="7" t="inlineStr">
         <is>
@@ -20349,7 +20349,7 @@
         </is>
       </c>
       <c r="C795" s="5" t="n">
-        <v>2025</v>
+        <v>2024</v>
       </c>
       <c r="D795" s="5" t="inlineStr">
         <is>
@@ -20374,7 +20374,7 @@
         </is>
       </c>
       <c r="C796" s="7" t="n">
-        <v>2026</v>
+        <v>2025</v>
       </c>
       <c r="D796" s="7" t="inlineStr">
         <is>
@@ -20390,7 +20390,7 @@
     <row r="797">
       <c r="A797" s="4" t="inlineStr">
         <is>
-          <t>Rock 'n' Roll Running Series Mexico City</t>
+          <t>Rock 'n' Roll Running Series Las Vegas</t>
         </is>
       </c>
       <c r="B797" s="5" t="inlineStr">
@@ -20399,7 +20399,7 @@
         </is>
       </c>
       <c r="C797" s="5" t="n">
-        <v>2025</v>
+        <v>2026</v>
       </c>
       <c r="D797" s="5" t="inlineStr">
         <is>
@@ -20415,7 +20415,7 @@
     <row r="798">
       <c r="A798" s="6" t="inlineStr">
         <is>
-          <t>Rock 'n' Roll Running Series San Diego</t>
+          <t>Rock 'n' Roll Running Series Mexico City</t>
         </is>
       </c>
       <c r="B798" s="7" t="inlineStr">
@@ -20449,23 +20449,23 @@
         </is>
       </c>
       <c r="C799" s="5" t="n">
-        <v>2026</v>
+        <v>2025</v>
       </c>
       <c r="D799" s="5" t="inlineStr">
         <is>
-          <t>1:04:18</t>
+          <t>N/A</t>
         </is>
       </c>
       <c r="E799" s="5" t="inlineStr">
         <is>
-          <t>1:16:00</t>
+          <t>N/A</t>
         </is>
       </c>
     </row>
     <row r="800">
       <c r="A800" s="6" t="inlineStr">
         <is>
-          <t>Royal Parks Half Marathon</t>
+          <t>Rock 'n' Roll Running Series San Diego</t>
         </is>
       </c>
       <c r="B800" s="7" t="inlineStr">
@@ -20474,23 +20474,23 @@
         </is>
       </c>
       <c r="C800" s="7" t="n">
-        <v>2025</v>
+        <v>2026</v>
       </c>
       <c r="D800" s="7" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>1:04:18</t>
         </is>
       </c>
       <c r="E800" s="7" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>1:16:00</t>
         </is>
       </c>
     </row>
     <row r="801">
       <c r="A801" s="4" t="inlineStr">
         <is>
-          <t>Run in Lyon (Semi)</t>
+          <t>Royal Parks Half Marathon</t>
         </is>
       </c>
       <c r="B801" s="5" t="inlineStr">
@@ -20499,7 +20499,7 @@
         </is>
       </c>
       <c r="C801" s="5" t="n">
-        <v>2023</v>
+        <v>2025</v>
       </c>
       <c r="D801" s="5" t="inlineStr">
         <is>
@@ -20524,16 +20524,16 @@
         </is>
       </c>
       <c r="C802" s="7" t="n">
-        <v>2024</v>
+        <v>2023</v>
       </c>
       <c r="D802" s="7" t="inlineStr">
         <is>
-          <t>1:05:44</t>
+          <t>N/A</t>
         </is>
       </c>
       <c r="E802" s="7" t="inlineStr">
         <is>
-          <t>1:18:34</t>
+          <t>N/A</t>
         </is>
       </c>
     </row>
@@ -20549,23 +20549,23 @@
         </is>
       </c>
       <c r="C803" s="5" t="n">
-        <v>2025</v>
+        <v>2024</v>
       </c>
       <c r="D803" s="5" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>1:05:44</t>
         </is>
       </c>
       <c r="E803" s="5" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>1:18:34</t>
         </is>
       </c>
     </row>
     <row r="804">
       <c r="A804" s="6" t="inlineStr">
         <is>
-          <t>Semi-Marathon de Boulogne-Billancourt</t>
+          <t>Run in Lyon (Semi)</t>
         </is>
       </c>
       <c r="B804" s="7" t="inlineStr">
@@ -20590,7 +20590,7 @@
     <row r="805">
       <c r="A805" s="4" t="inlineStr">
         <is>
-          <t>St. Jude Rock 'n' Roll Running Series Washington DC</t>
+          <t>Semi-Marathon de Boulogne-Billancourt</t>
         </is>
       </c>
       <c r="B805" s="5" t="inlineStr">
@@ -20615,7 +20615,7 @@
     <row r="806">
       <c r="A806" s="6" t="inlineStr">
         <is>
-          <t>St. Jude Rock 'n' Roll Series Nashville</t>
+          <t>St. Jude Rock 'n' Roll Running Series Washington DC</t>
         </is>
       </c>
       <c r="B806" s="7" t="inlineStr">
@@ -20640,7 +20640,7 @@
     <row r="807">
       <c r="A807" s="4" t="inlineStr">
         <is>
-          <t>Standard Chartered Hong Kong Half Marathon</t>
+          <t>St. Jude Rock 'n' Roll Series Nashville</t>
         </is>
       </c>
       <c r="B807" s="5" t="inlineStr">
@@ -20649,16 +20649,16 @@
         </is>
       </c>
       <c r="C807" s="5" t="n">
-        <v>2019</v>
+        <v>2025</v>
       </c>
       <c r="D807" s="5" t="inlineStr">
         <is>
-          <t>1:01:13</t>
+          <t>N/A</t>
         </is>
       </c>
       <c r="E807" s="5" t="inlineStr">
         <is>
-          <t>1:09:28</t>
+          <t>N/A</t>
         </is>
       </c>
     </row>
@@ -20674,16 +20674,16 @@
         </is>
       </c>
       <c r="C808" s="7" t="n">
-        <v>2025</v>
+        <v>2019</v>
       </c>
       <c r="D808" s="7" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>1:01:13</t>
         </is>
       </c>
       <c r="E808" s="7" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>1:09:28</t>
         </is>
       </c>
     </row>
@@ -20699,7 +20699,7 @@
         </is>
       </c>
       <c r="C809" s="5" t="n">
-        <v>2026</v>
+        <v>2025</v>
       </c>
       <c r="D809" s="5" t="inlineStr">
         <is>
@@ -20715,7 +20715,7 @@
     <row r="810">
       <c r="A810" s="6" t="inlineStr">
         <is>
-          <t>Standard Chartered KL Half Marathon</t>
+          <t>Standard Chartered Hong Kong Half Marathon</t>
         </is>
       </c>
       <c r="B810" s="7" t="inlineStr">
@@ -20724,23 +20724,23 @@
         </is>
       </c>
       <c r="C810" s="7" t="n">
-        <v>2025</v>
+        <v>2026</v>
       </c>
       <c r="D810" s="7" t="inlineStr">
         <is>
-          <t>1:11:08</t>
+          <t>N/A</t>
         </is>
       </c>
       <c r="E810" s="7" t="inlineStr">
         <is>
-          <t>1:23:55</t>
+          <t>N/A</t>
         </is>
       </c>
     </row>
     <row r="811">
       <c r="A811" s="4" t="inlineStr">
         <is>
-          <t>Standard Chartered Singapore Half Marathon</t>
+          <t>Standard Chartered KL Half Marathon</t>
         </is>
       </c>
       <c r="B811" s="5" t="inlineStr">
@@ -20753,19 +20753,19 @@
       </c>
       <c r="D811" s="5" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>1:11:08</t>
         </is>
       </c>
       <c r="E811" s="5" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>1:23:55</t>
         </is>
       </c>
     </row>
     <row r="812">
       <c r="A812" s="6" t="inlineStr">
         <is>
-          <t>TCS Mizuno Half Marathon</t>
+          <t>Standard Chartered Singapore Half Marathon</t>
         </is>
       </c>
       <c r="B812" s="7" t="inlineStr">
@@ -20774,16 +20774,16 @@
         </is>
       </c>
       <c r="C812" s="7" t="n">
-        <v>2023</v>
+        <v>2025</v>
       </c>
       <c r="D812" s="7" t="inlineStr">
         <is>
-          <t>1:05:23</t>
+          <t>N/A</t>
         </is>
       </c>
       <c r="E812" s="7" t="inlineStr">
         <is>
-          <t>1:13:59</t>
+          <t>N/A</t>
         </is>
       </c>
     </row>
@@ -20799,16 +20799,16 @@
         </is>
       </c>
       <c r="C813" s="5" t="n">
-        <v>2024</v>
+        <v>2023</v>
       </c>
       <c r="D813" s="5" t="inlineStr">
         <is>
-          <t>1:06:28</t>
+          <t>1:05:23</t>
         </is>
       </c>
       <c r="E813" s="5" t="inlineStr">
         <is>
-          <t>1:17:54</t>
+          <t>1:13:59</t>
         </is>
       </c>
     </row>
@@ -20824,16 +20824,16 @@
         </is>
       </c>
       <c r="C814" s="7" t="n">
-        <v>2025</v>
+        <v>2024</v>
       </c>
       <c r="D814" s="7" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>1:06:28</t>
         </is>
       </c>
       <c r="E814" s="7" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>1:17:54</t>
         </is>
       </c>
     </row>
@@ -20853,19 +20853,19 @@
       </c>
       <c r="D815" s="5" t="inlineStr">
         <is>
-          <t>1:04:21</t>
+          <t>N/A</t>
         </is>
       </c>
       <c r="E815" s="5" t="inlineStr">
         <is>
-          <t>1:10:02</t>
+          <t>N/A</t>
         </is>
       </c>
     </row>
     <row r="816">
       <c r="A816" s="6" t="inlineStr">
         <is>
-          <t>TCS Toronto Waterfront Marathon (Half)</t>
+          <t>TCS Mizuno Half Marathon</t>
         </is>
       </c>
       <c r="B816" s="7" t="inlineStr">
@@ -20874,16 +20874,16 @@
         </is>
       </c>
       <c r="C816" s="7" t="n">
-        <v>2023</v>
+        <v>2025</v>
       </c>
       <c r="D816" s="7" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>1:04:21</t>
         </is>
       </c>
       <c r="E816" s="7" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>1:10:02</t>
         </is>
       </c>
     </row>
@@ -20899,7 +20899,7 @@
         </is>
       </c>
       <c r="C817" s="5" t="n">
-        <v>2024</v>
+        <v>2023</v>
       </c>
       <c r="D817" s="5" t="inlineStr">
         <is>
@@ -20924,7 +20924,7 @@
         </is>
       </c>
       <c r="C818" s="7" t="n">
-        <v>2025</v>
+        <v>2024</v>
       </c>
       <c r="D818" s="7" t="inlineStr">
         <is>
@@ -20940,7 +20940,7 @@
     <row r="819">
       <c r="A819" s="4" t="inlineStr">
         <is>
-          <t>Taipei Half Marathon</t>
+          <t>TCS Toronto Waterfront Marathon (Half)</t>
         </is>
       </c>
       <c r="B819" s="5" t="inlineStr">
@@ -20949,7 +20949,7 @@
         </is>
       </c>
       <c r="C819" s="5" t="n">
-        <v>2023</v>
+        <v>2025</v>
       </c>
       <c r="D819" s="5" t="inlineStr">
         <is>
@@ -20974,7 +20974,7 @@
         </is>
       </c>
       <c r="C820" s="7" t="n">
-        <v>2024</v>
+        <v>2023</v>
       </c>
       <c r="D820" s="7" t="inlineStr">
         <is>
@@ -20999,7 +20999,7 @@
         </is>
       </c>
       <c r="C821" s="5" t="n">
-        <v>2025</v>
+        <v>2024</v>
       </c>
       <c r="D821" s="5" t="inlineStr">
         <is>
@@ -21015,7 +21015,7 @@
     <row r="822">
       <c r="A822" s="6" t="inlineStr">
         <is>
-          <t>Tata Mumbai Marathon (Half)</t>
+          <t>Taipei Half Marathon</t>
         </is>
       </c>
       <c r="B822" s="7" t="inlineStr">
@@ -21049,7 +21049,7 @@
         </is>
       </c>
       <c r="C823" s="5" t="n">
-        <v>2026</v>
+        <v>2025</v>
       </c>
       <c r="D823" s="5" t="inlineStr">
         <is>
@@ -21065,7 +21065,7 @@
     <row r="824">
       <c r="A824" s="6" t="inlineStr">
         <is>
-          <t>The Big Half</t>
+          <t>Tata Mumbai Marathon (Half)</t>
         </is>
       </c>
       <c r="B824" s="7" t="inlineStr">
@@ -21074,7 +21074,7 @@
         </is>
       </c>
       <c r="C824" s="7" t="n">
-        <v>2025</v>
+        <v>2026</v>
       </c>
       <c r="D824" s="7" t="inlineStr">
         <is>
@@ -21090,7 +21090,7 @@
     <row r="825">
       <c r="A825" s="4" t="inlineStr">
         <is>
-          <t>Tokyo Legacy Half Marathon</t>
+          <t>The Big Half</t>
         </is>
       </c>
       <c r="B825" s="5" t="inlineStr">
@@ -21115,7 +21115,7 @@
     <row r="826">
       <c r="A826" s="6" t="inlineStr">
         <is>
-          <t>United Airlines NYC Half</t>
+          <t>Tokyo Legacy Half Marathon</t>
         </is>
       </c>
       <c r="B826" s="7" t="inlineStr">
@@ -21124,16 +21124,16 @@
         </is>
       </c>
       <c r="C826" s="7" t="n">
-        <v>2006</v>
+        <v>2025</v>
       </c>
       <c r="D826" s="7" t="inlineStr">
         <is>
-          <t>1:01:22</t>
+          <t>N/A</t>
         </is>
       </c>
       <c r="E826" s="7" t="inlineStr">
         <is>
-          <t>1:09:43</t>
+          <t>N/A</t>
         </is>
       </c>
     </row>
@@ -21149,16 +21149,16 @@
         </is>
       </c>
       <c r="C827" s="5" t="n">
-        <v>2007</v>
+        <v>2006</v>
       </c>
       <c r="D827" s="5" t="inlineStr">
         <is>
-          <t>0:59:24</t>
+          <t>1:01:22</t>
         </is>
       </c>
       <c r="E827" s="5" t="inlineStr">
         <is>
-          <t>1:10:32</t>
+          <t>1:09:43</t>
         </is>
       </c>
     </row>
@@ -21174,16 +21174,16 @@
         </is>
       </c>
       <c r="C828" s="7" t="n">
-        <v>2008</v>
+        <v>2007</v>
       </c>
       <c r="D828" s="7" t="inlineStr">
         <is>
-          <t>1:00:58</t>
+          <t>0:59:24</t>
         </is>
       </c>
       <c r="E828" s="7" t="inlineStr">
         <is>
-          <t>1:10:19</t>
+          <t>1:10:32</t>
         </is>
       </c>
     </row>
@@ -21199,16 +21199,16 @@
         </is>
       </c>
       <c r="C829" s="5" t="n">
-        <v>2009</v>
+        <v>2008</v>
       </c>
       <c r="D829" s="5" t="inlineStr">
         <is>
-          <t>1:01:06</t>
+          <t>1:00:58</t>
         </is>
       </c>
       <c r="E829" s="5" t="inlineStr">
         <is>
-          <t>1:09:32</t>
+          <t>1:10:19</t>
         </is>
       </c>
     </row>
@@ -21224,16 +21224,16 @@
         </is>
       </c>
       <c r="C830" s="7" t="n">
-        <v>2010</v>
+        <v>2009</v>
       </c>
       <c r="D830" s="7" t="inlineStr">
         <is>
-          <t>0:59:52</t>
+          <t>1:01:06</t>
         </is>
       </c>
       <c r="E830" s="7" t="inlineStr">
         <is>
-          <t>1:09:25</t>
+          <t>1:09:32</t>
         </is>
       </c>
     </row>
@@ -21249,16 +21249,16 @@
         </is>
       </c>
       <c r="C831" s="5" t="n">
-        <v>2011</v>
+        <v>2010</v>
       </c>
       <c r="D831" s="5" t="inlineStr">
         <is>
-          <t>1:00:23</t>
+          <t>0:59:52</t>
         </is>
       </c>
       <c r="E831" s="5" t="inlineStr">
         <is>
-          <t>1:08:52</t>
+          <t>1:09:25</t>
         </is>
       </c>
     </row>
@@ -21274,16 +21274,16 @@
         </is>
       </c>
       <c r="C832" s="7" t="n">
-        <v>2012</v>
+        <v>2011</v>
       </c>
       <c r="D832" s="7" t="inlineStr">
         <is>
-          <t>0:59:39</t>
+          <t>1:00:23</t>
         </is>
       </c>
       <c r="E832" s="7" t="inlineStr">
         <is>
-          <t>1:08:35</t>
+          <t>1:08:52</t>
         </is>
       </c>
     </row>
@@ -21299,16 +21299,16 @@
         </is>
       </c>
       <c r="C833" s="5" t="n">
-        <v>2013</v>
+        <v>2012</v>
       </c>
       <c r="D833" s="5" t="inlineStr">
         <is>
-          <t>1:01:02</t>
+          <t>0:59:39</t>
         </is>
       </c>
       <c r="E833" s="5" t="inlineStr">
         <is>
-          <t>1:09:09</t>
+          <t>1:08:35</t>
         </is>
       </c>
     </row>
@@ -21324,16 +21324,16 @@
         </is>
       </c>
       <c r="C834" s="7" t="n">
-        <v>2014</v>
+        <v>2013</v>
       </c>
       <c r="D834" s="7" t="inlineStr">
         <is>
-          <t>1:00:50</t>
+          <t>1:01:02</t>
         </is>
       </c>
       <c r="E834" s="7" t="inlineStr">
         <is>
-          <t>1:08:31</t>
+          <t>1:09:09</t>
         </is>
       </c>
     </row>
@@ -21349,16 +21349,16 @@
         </is>
       </c>
       <c r="C835" s="5" t="n">
-        <v>2025</v>
+        <v>2014</v>
       </c>
       <c r="D835" s="5" t="inlineStr">
         <is>
-          <t>1:01:31</t>
+          <t>1:00:50</t>
         </is>
       </c>
       <c r="E835" s="5" t="inlineStr">
         <is>
-          <t>1:07:04</t>
+          <t>1:08:31</t>
         </is>
       </c>
     </row>
@@ -21374,23 +21374,23 @@
         </is>
       </c>
       <c r="C836" s="7" t="n">
-        <v>2026</v>
+        <v>2025</v>
       </c>
       <c r="D836" s="7" t="inlineStr">
         <is>
-          <t>0:59:30</t>
+          <t>1:01:31</t>
         </is>
       </c>
       <c r="E836" s="7" t="inlineStr">
         <is>
-          <t>1:06:33</t>
+          <t>1:07:04</t>
         </is>
       </c>
     </row>
     <row r="837">
       <c r="A837" s="4" t="inlineStr">
         <is>
-          <t>Valencia Half Marathon Trinidad Alfonso Zurich</t>
+          <t>United Airlines NYC Half</t>
         </is>
       </c>
       <c r="B837" s="5" t="inlineStr">
@@ -21399,23 +21399,23 @@
         </is>
       </c>
       <c r="C837" s="5" t="n">
-        <v>2025</v>
+        <v>2026</v>
       </c>
       <c r="D837" s="5" t="inlineStr">
         <is>
-          <t>0:58:02</t>
+          <t>0:59:30</t>
         </is>
       </c>
       <c r="E837" s="5" t="inlineStr">
         <is>
-          <t>1:03:08</t>
+          <t>1:06:33</t>
         </is>
       </c>
     </row>
     <row r="838">
       <c r="A838" s="6" t="inlineStr">
         <is>
-          <t>Vedanta Delhi Half Marathon</t>
+          <t>Valencia Half Marathon Trinidad Alfonso Zurich</t>
         </is>
       </c>
       <c r="B838" s="7" t="inlineStr">
@@ -21428,19 +21428,19 @@
       </c>
       <c r="D838" s="7" t="inlineStr">
         <is>
-          <t>0:59:50</t>
+          <t>0:58:02</t>
         </is>
       </c>
       <c r="E838" s="7" t="inlineStr">
         <is>
-          <t>1:07:20</t>
+          <t>1:03:08</t>
         </is>
       </c>
     </row>
     <row r="839">
       <c r="A839" s="4" t="inlineStr">
         <is>
-          <t>Vienna City Half Marathon</t>
+          <t>Vedanta Delhi Half Marathon</t>
         </is>
       </c>
       <c r="B839" s="5" t="inlineStr">
@@ -21453,19 +21453,19 @@
       </c>
       <c r="D839" s="5" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>0:59:50</t>
         </is>
       </c>
       <c r="E839" s="5" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>1:07:20</t>
         </is>
       </c>
     </row>
     <row r="840">
       <c r="A840" s="6" t="inlineStr">
         <is>
-          <t>Walt Disney World Marathon Weekend</t>
+          <t>Vienna City Half Marathon</t>
         </is>
       </c>
       <c r="B840" s="7" t="inlineStr">
@@ -21499,7 +21499,7 @@
         </is>
       </c>
       <c r="C841" s="5" t="n">
-        <v>2026</v>
+        <v>2025</v>
       </c>
       <c r="D841" s="5" t="inlineStr">
         <is>
@@ -21515,7 +21515,7 @@
     <row r="842">
       <c r="A842" s="6" t="inlineStr">
         <is>
-          <t>Warsaw Half Marathon</t>
+          <t>Walt Disney World Marathon Weekend</t>
         </is>
       </c>
       <c r="B842" s="7" t="inlineStr">
@@ -21524,7 +21524,7 @@
         </is>
       </c>
       <c r="C842" s="7" t="n">
-        <v>2024</v>
+        <v>2026</v>
       </c>
       <c r="D842" s="7" t="inlineStr">
         <is>
@@ -21549,7 +21549,7 @@
         </is>
       </c>
       <c r="C843" s="5" t="n">
-        <v>2025</v>
+        <v>2024</v>
       </c>
       <c r="D843" s="5" t="inlineStr">
         <is>
@@ -21565,7 +21565,7 @@
     <row r="844">
       <c r="A844" s="6" t="inlineStr">
         <is>
-          <t>Wizz Air Rome Half Marathon by Brooks</t>
+          <t>Warsaw Half Marathon</t>
         </is>
       </c>
       <c r="B844" s="7" t="inlineStr">
@@ -21590,7 +21590,7 @@
     <row r="845">
       <c r="A845" s="4" t="inlineStr">
         <is>
-          <t>Zurich Rock 'n' Roll Running Series Madrid (Half)</t>
+          <t>Wizz Air Rome Half Marathon by Brooks</t>
         </is>
       </c>
       <c r="B845" s="5" t="inlineStr">
@@ -21599,7 +21599,7 @@
         </is>
       </c>
       <c r="C845" s="5" t="n">
-        <v>2023</v>
+        <v>2025</v>
       </c>
       <c r="D845" s="5" t="inlineStr">
         <is>
@@ -21624,7 +21624,7 @@
         </is>
       </c>
       <c r="C846" s="7" t="n">
-        <v>2024</v>
+        <v>2023</v>
       </c>
       <c r="D846" s="7" t="inlineStr">
         <is>
@@ -21649,41 +21649,41 @@
         </is>
       </c>
       <c r="C847" s="5" t="n">
+        <v>2024</v>
+      </c>
+      <c r="D847" s="5" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="E847" s="5" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+    </row>
+    <row r="848">
+      <c r="A848" s="6" t="inlineStr">
+        <is>
+          <t>Zurich Rock 'n' Roll Running Series Madrid (Half)</t>
+        </is>
+      </c>
+      <c r="B848" s="7" t="inlineStr">
+        <is>
+          <t>21K</t>
+        </is>
+      </c>
+      <c r="C848" s="7" t="n">
         <v>2025</v>
       </c>
-      <c r="D847" s="5" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="E847" s="5" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-    </row>
-    <row r="848">
-      <c r="A848" s="8" t="inlineStr">
-        <is>
-          <t>10K Montmartre</t>
-        </is>
-      </c>
-      <c r="B848" s="9" t="inlineStr">
-        <is>
-          <t>10K</t>
-        </is>
-      </c>
-      <c r="C848" s="9" t="n">
-        <v>2025</v>
-      </c>
-      <c r="D848" s="9" t="inlineStr">
-        <is>
-          <t>0:31:14</t>
-        </is>
-      </c>
-      <c r="E848" s="9" t="inlineStr">
-        <is>
-          <t>0:35:46</t>
+      <c r="D848" s="7" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="E848" s="7" t="inlineStr">
+        <is>
+          <t>N/A</t>
         </is>
       </c>
     </row>
@@ -21699,23 +21699,23 @@
         </is>
       </c>
       <c r="C849" s="5" t="n">
-        <v>2026</v>
+        <v>2025</v>
       </c>
       <c r="D849" s="5" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>0:31:14</t>
         </is>
       </c>
       <c r="E849" s="5" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>0:35:46</t>
         </is>
       </c>
     </row>
     <row r="850">
       <c r="A850" s="8" t="inlineStr">
         <is>
-          <t>10K Valencia Ibercaja by Kiprun</t>
+          <t>10K Montmartre</t>
         </is>
       </c>
       <c r="B850" s="9" t="inlineStr">
@@ -21724,7 +21724,7 @@
         </is>
       </c>
       <c r="C850" s="9" t="n">
-        <v>2023</v>
+        <v>2026</v>
       </c>
       <c r="D850" s="9" t="inlineStr">
         <is>
@@ -21733,7 +21733,7 @@
       </c>
       <c r="E850" s="9" t="inlineStr">
         <is>
-          <t>0:29:19</t>
+          <t>N/A</t>
         </is>
       </c>
     </row>
@@ -21749,7 +21749,7 @@
         </is>
       </c>
       <c r="C851" s="5" t="n">
-        <v>2024</v>
+        <v>2023</v>
       </c>
       <c r="D851" s="5" t="inlineStr">
         <is>
@@ -21758,7 +21758,7 @@
       </c>
       <c r="E851" s="5" t="inlineStr">
         <is>
-          <t>0:28:45</t>
+          <t>0:29:19</t>
         </is>
       </c>
     </row>
@@ -21774,7 +21774,7 @@
         </is>
       </c>
       <c r="C852" s="9" t="n">
-        <v>2025</v>
+        <v>2024</v>
       </c>
       <c r="D852" s="9" t="inlineStr">
         <is>
@@ -21783,7 +21783,7 @@
       </c>
       <c r="E852" s="9" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>0:28:45</t>
         </is>
       </c>
     </row>
@@ -21799,23 +21799,23 @@
         </is>
       </c>
       <c r="C853" s="5" t="n">
-        <v>2026</v>
+        <v>2025</v>
       </c>
       <c r="D853" s="5" t="inlineStr">
         <is>
-          <t>0:26:45</t>
+          <t>N/A</t>
         </is>
       </c>
       <c r="E853" s="5" t="inlineStr">
         <is>
-          <t>0:29:25</t>
+          <t>N/A</t>
         </is>
       </c>
     </row>
     <row r="854">
       <c r="A854" s="8" t="inlineStr">
         <is>
-          <t>10km Fulfil des Champs Elysées</t>
+          <t>10K Valencia Ibercaja by Kiprun</t>
         </is>
       </c>
       <c r="B854" s="9" t="inlineStr">
@@ -21828,19 +21828,19 @@
       </c>
       <c r="D854" s="9" t="inlineStr">
         <is>
-          <t>0:28:34</t>
+          <t>0:26:45</t>
         </is>
       </c>
       <c r="E854" s="9" t="inlineStr">
         <is>
-          <t>0:33:24</t>
+          <t>0:29:25</t>
         </is>
       </c>
     </row>
     <row r="855">
       <c r="A855" s="4" t="inlineStr">
         <is>
-          <t>AJ Bell Great Birmingham Run 10K</t>
+          <t>10km Fulfil des Champs Elysées</t>
         </is>
       </c>
       <c r="B855" s="5" t="inlineStr">
@@ -21849,23 +21849,23 @@
         </is>
       </c>
       <c r="C855" s="5" t="n">
-        <v>2025</v>
+        <v>2026</v>
       </c>
       <c r="D855" s="5" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>0:28:34</t>
         </is>
       </c>
       <c r="E855" s="5" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>0:33:24</t>
         </is>
       </c>
     </row>
     <row r="856">
       <c r="A856" s="8" t="inlineStr">
         <is>
-          <t>AJ Bell Great Bristol Run 10K</t>
+          <t>AJ Bell Great Birmingham Run 10K</t>
         </is>
       </c>
       <c r="B856" s="9" t="inlineStr">
@@ -21899,23 +21899,23 @@
         </is>
       </c>
       <c r="C857" s="5" t="n">
-        <v>2026</v>
+        <v>2025</v>
       </c>
       <c r="D857" s="5" t="inlineStr">
         <is>
-          <t>0:30:55</t>
+          <t>N/A</t>
         </is>
       </c>
       <c r="E857" s="5" t="inlineStr">
         <is>
-          <t>0:36:50</t>
+          <t>N/A</t>
         </is>
       </c>
     </row>
     <row r="858">
       <c r="A858" s="8" t="inlineStr">
         <is>
-          <t>AJ Bell Great Manchester Run</t>
+          <t>AJ Bell Great Bristol Run 10K</t>
         </is>
       </c>
       <c r="B858" s="9" t="inlineStr">
@@ -21924,16 +21924,16 @@
         </is>
       </c>
       <c r="C858" s="9" t="n">
-        <v>2021</v>
+        <v>2026</v>
       </c>
       <c r="D858" s="9" t="inlineStr">
         <is>
-          <t>0:28:03</t>
+          <t>0:30:55</t>
         </is>
       </c>
       <c r="E858" s="9" t="inlineStr">
         <is>
-          <t>0:30:51</t>
+          <t>0:36:50</t>
         </is>
       </c>
     </row>
@@ -21949,23 +21949,23 @@
         </is>
       </c>
       <c r="C859" s="5" t="n">
-        <v>2025</v>
+        <v>2021</v>
       </c>
       <c r="D859" s="5" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>0:28:03</t>
         </is>
       </c>
       <c r="E859" s="5" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>0:30:51</t>
         </is>
       </c>
     </row>
     <row r="860">
       <c r="A860" s="8" t="inlineStr">
         <is>
-          <t>AJ Bell Great Manchester Run (10K)</t>
+          <t>AJ Bell Great Manchester Run</t>
         </is>
       </c>
       <c r="B860" s="9" t="inlineStr">
@@ -21974,7 +21974,7 @@
         </is>
       </c>
       <c r="C860" s="9" t="n">
-        <v>2024</v>
+        <v>2025</v>
       </c>
       <c r="D860" s="9" t="inlineStr">
         <is>
@@ -21999,7 +21999,7 @@
         </is>
       </c>
       <c r="C861" s="5" t="n">
-        <v>2025</v>
+        <v>2024</v>
       </c>
       <c r="D861" s="5" t="inlineStr">
         <is>
@@ -22015,7 +22015,7 @@
     <row r="862">
       <c r="A862" s="8" t="inlineStr">
         <is>
-          <t>AJ Bell Great North 10K</t>
+          <t>AJ Bell Great Manchester Run (10K)</t>
         </is>
       </c>
       <c r="B862" s="9" t="inlineStr">
@@ -22040,7 +22040,7 @@
     <row r="863">
       <c r="A863" s="4" t="inlineStr">
         <is>
-          <t>ASICS LDNX</t>
+          <t>AJ Bell Great North 10K</t>
         </is>
       </c>
       <c r="B863" s="5" t="inlineStr">
@@ -22065,7 +22065,7 @@
     <row r="864">
       <c r="A864" s="8" t="inlineStr">
         <is>
-          <t>Adidas 10K Paris</t>
+          <t>ASICS LDNX</t>
         </is>
       </c>
       <c r="B864" s="9" t="inlineStr">
@@ -22074,7 +22074,7 @@
         </is>
       </c>
       <c r="C864" s="9" t="n">
-        <v>2023</v>
+        <v>2025</v>
       </c>
       <c r="D864" s="9" t="inlineStr">
         <is>
@@ -22099,16 +22099,16 @@
         </is>
       </c>
       <c r="C865" s="5" t="n">
-        <v>2024</v>
+        <v>2023</v>
       </c>
       <c r="D865" s="5" t="inlineStr">
         <is>
-          <t>0:29:37</t>
+          <t>N/A</t>
         </is>
       </c>
       <c r="E865" s="5" t="inlineStr">
         <is>
-          <t>0:32:18</t>
+          <t>N/A</t>
         </is>
       </c>
     </row>
@@ -22124,16 +22124,16 @@
         </is>
       </c>
       <c r="C866" s="9" t="n">
-        <v>2025</v>
+        <v>2024</v>
       </c>
       <c r="D866" s="9" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>0:29:37</t>
         </is>
       </c>
       <c r="E866" s="9" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>0:32:18</t>
         </is>
       </c>
     </row>
@@ -22149,23 +22149,23 @@
         </is>
       </c>
       <c r="C867" s="5" t="n">
-        <v>2026</v>
+        <v>2025</v>
       </c>
       <c r="D867" s="5" t="inlineStr">
         <is>
-          <t>0:28:11</t>
+          <t>N/A</t>
         </is>
       </c>
       <c r="E867" s="5" t="inlineStr">
         <is>
-          <t>0:31:48</t>
+          <t>N/A</t>
         </is>
       </c>
     </row>
     <row r="868">
       <c r="A868" s="8" t="inlineStr">
         <is>
-          <t>Atlanta Journal-Constitution Peachtree Road Race</t>
+          <t>Adidas 10K Paris</t>
         </is>
       </c>
       <c r="B868" s="9" t="inlineStr">
@@ -22174,16 +22174,16 @@
         </is>
       </c>
       <c r="C868" s="9" t="n">
-        <v>2023</v>
+        <v>2026</v>
       </c>
       <c r="D868" s="9" t="inlineStr">
         <is>
-          <t>0:27:41</t>
+          <t>0:28:11</t>
         </is>
       </c>
       <c r="E868" s="9" t="inlineStr">
         <is>
-          <t>0:30:43</t>
+          <t>0:31:48</t>
         </is>
       </c>
     </row>
@@ -22199,16 +22199,16 @@
         </is>
       </c>
       <c r="C869" s="5" t="n">
-        <v>2024</v>
+        <v>2023</v>
       </c>
       <c r="D869" s="5" t="inlineStr">
         <is>
-          <t>0:28:03</t>
+          <t>0:27:41</t>
         </is>
       </c>
       <c r="E869" s="5" t="inlineStr">
         <is>
-          <t>0:31:12</t>
+          <t>0:30:43</t>
         </is>
       </c>
     </row>
@@ -22224,23 +22224,23 @@
         </is>
       </c>
       <c r="C870" s="9" t="n">
-        <v>2025</v>
+        <v>2024</v>
       </c>
       <c r="D870" s="9" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>0:28:03</t>
         </is>
       </c>
       <c r="E870" s="9" t="inlineStr">
         <is>
-          <t>0:31:29</t>
+          <t>0:31:12</t>
         </is>
       </c>
     </row>
     <row r="871">
       <c r="A871" s="4" t="inlineStr">
         <is>
-          <t>BOLDERBoulder 10K</t>
+          <t>Atlanta Journal-Constitution Peachtree Road Race</t>
         </is>
       </c>
       <c r="B871" s="5" t="inlineStr">
@@ -22249,16 +22249,16 @@
         </is>
       </c>
       <c r="C871" s="5" t="n">
-        <v>2023</v>
+        <v>2025</v>
       </c>
       <c r="D871" s="5" t="inlineStr">
         <is>
-          <t>0:29:08</t>
+          <t>N/A</t>
         </is>
       </c>
       <c r="E871" s="5" t="inlineStr">
         <is>
-          <t>0:33:25</t>
+          <t>0:31:29</t>
         </is>
       </c>
     </row>
@@ -22274,16 +22274,16 @@
         </is>
       </c>
       <c r="C872" s="9" t="n">
-        <v>2024</v>
+        <v>2023</v>
       </c>
       <c r="D872" s="9" t="inlineStr">
         <is>
-          <t>0:29:13</t>
+          <t>0:29:08</t>
         </is>
       </c>
       <c r="E872" s="9" t="inlineStr">
         <is>
-          <t>0:32:45</t>
+          <t>0:33:25</t>
         </is>
       </c>
     </row>
@@ -22299,16 +22299,16 @@
         </is>
       </c>
       <c r="C873" s="5" t="n">
-        <v>2025</v>
+        <v>2024</v>
       </c>
       <c r="D873" s="5" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>0:29:13</t>
         </is>
       </c>
       <c r="E873" s="5" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>0:32:45</t>
         </is>
       </c>
     </row>
@@ -22328,19 +22328,19 @@
       </c>
       <c r="D874" s="9" t="inlineStr">
         <is>
-          <t>0:28:36</t>
+          <t>N/A</t>
         </is>
       </c>
       <c r="E874" s="9" t="inlineStr">
         <is>
-          <t>0:31:51</t>
+          <t>N/A</t>
         </is>
       </c>
     </row>
     <row r="875">
       <c r="A875" s="4" t="inlineStr">
         <is>
-          <t>Bangsaen10</t>
+          <t>BOLDERBoulder 10K</t>
         </is>
       </c>
       <c r="B875" s="5" t="inlineStr">
@@ -22349,16 +22349,16 @@
         </is>
       </c>
       <c r="C875" s="5" t="n">
-        <v>2023</v>
+        <v>2025</v>
       </c>
       <c r="D875" s="5" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>0:28:36</t>
         </is>
       </c>
       <c r="E875" s="5" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>0:31:51</t>
         </is>
       </c>
     </row>
@@ -22374,7 +22374,7 @@
         </is>
       </c>
       <c r="C876" s="9" t="n">
-        <v>2024</v>
+        <v>2023</v>
       </c>
       <c r="D876" s="9" t="inlineStr">
         <is>
@@ -22399,7 +22399,7 @@
         </is>
       </c>
       <c r="C877" s="5" t="n">
-        <v>2025</v>
+        <v>2024</v>
       </c>
       <c r="D877" s="5" t="inlineStr">
         <is>
@@ -22415,7 +22415,7 @@
     <row r="878">
       <c r="A878" s="8" t="inlineStr">
         <is>
-          <t>Cancer Research UK London Winter Run</t>
+          <t>Bangsaen10</t>
         </is>
       </c>
       <c r="B878" s="9" t="inlineStr">
@@ -22424,16 +22424,16 @@
         </is>
       </c>
       <c r="C878" s="9" t="n">
-        <v>2023</v>
+        <v>2025</v>
       </c>
       <c r="D878" s="9" t="inlineStr">
         <is>
-          <t>0:28:52</t>
+          <t>N/A</t>
         </is>
       </c>
       <c r="E878" s="9" t="inlineStr">
         <is>
-          <t>0:31:59</t>
+          <t>N/A</t>
         </is>
       </c>
     </row>
@@ -22449,16 +22449,16 @@
         </is>
       </c>
       <c r="C879" s="5" t="n">
-        <v>2024</v>
+        <v>2023</v>
       </c>
       <c r="D879" s="5" t="inlineStr">
         <is>
-          <t>0:28:46</t>
+          <t>0:28:52</t>
         </is>
       </c>
       <c r="E879" s="5" t="inlineStr">
         <is>
-          <t>0:32:33</t>
+          <t>0:31:59</t>
         </is>
       </c>
     </row>
@@ -22474,16 +22474,16 @@
         </is>
       </c>
       <c r="C880" s="9" t="n">
-        <v>2025</v>
+        <v>2024</v>
       </c>
       <c r="D880" s="9" t="inlineStr">
         <is>
-          <t>0:29:22</t>
+          <t>0:28:46</t>
         </is>
       </c>
       <c r="E880" s="9" t="inlineStr">
         <is>
-          <t>0:34:32</t>
+          <t>0:32:33</t>
         </is>
       </c>
     </row>
@@ -22499,23 +22499,23 @@
         </is>
       </c>
       <c r="C881" s="5" t="n">
-        <v>2026</v>
+        <v>2025</v>
       </c>
       <c r="D881" s="5" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>0:29:22</t>
         </is>
       </c>
       <c r="E881" s="5" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>0:34:32</t>
         </is>
       </c>
     </row>
     <row r="882">
       <c r="A882" s="8" t="inlineStr">
         <is>
-          <t>Cooper River Bridge Run</t>
+          <t>Cancer Research UK London Winter Run</t>
         </is>
       </c>
       <c r="B882" s="9" t="inlineStr">
@@ -22524,7 +22524,7 @@
         </is>
       </c>
       <c r="C882" s="9" t="n">
-        <v>2023</v>
+        <v>2026</v>
       </c>
       <c r="D882" s="9" t="inlineStr">
         <is>
@@ -22549,7 +22549,7 @@
         </is>
       </c>
       <c r="C883" s="5" t="n">
-        <v>2024</v>
+        <v>2023</v>
       </c>
       <c r="D883" s="5" t="inlineStr">
         <is>
@@ -22574,16 +22574,16 @@
         </is>
       </c>
       <c r="C884" s="9" t="n">
-        <v>2025</v>
+        <v>2024</v>
       </c>
       <c r="D884" s="9" t="inlineStr">
         <is>
-          <t>0:28:27</t>
+          <t>N/A</t>
         </is>
       </c>
       <c r="E884" s="9" t="inlineStr">
         <is>
-          <t>0:31:49</t>
+          <t>N/A</t>
         </is>
       </c>
     </row>
@@ -22603,19 +22603,19 @@
       </c>
       <c r="D885" s="5" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>0:28:27</t>
         </is>
       </c>
       <c r="E885" s="5" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>0:31:49</t>
         </is>
       </c>
     </row>
     <row r="886">
       <c r="A886" s="8" t="inlineStr">
         <is>
-          <t>Cursa El corte Ingles</t>
+          <t>Cooper River Bridge Run</t>
         </is>
       </c>
       <c r="B886" s="9" t="inlineStr">
@@ -22624,23 +22624,23 @@
         </is>
       </c>
       <c r="C886" s="9" t="n">
-        <v>2026</v>
+        <v>2025</v>
       </c>
       <c r="D886" s="9" t="inlineStr">
         <is>
-          <t>0:29:44</t>
+          <t>N/A</t>
         </is>
       </c>
       <c r="E886" s="9" t="inlineStr">
         <is>
-          <t>0:35:28</t>
+          <t>N/A</t>
         </is>
       </c>
     </row>
     <row r="887">
       <c r="A887" s="4" t="inlineStr">
         <is>
-          <t>EDP Meia Maratona de Lisboa - Vodafone 10K</t>
+          <t>Cursa El corte Ingles</t>
         </is>
       </c>
       <c r="B887" s="5" t="inlineStr">
@@ -22649,16 +22649,16 @@
         </is>
       </c>
       <c r="C887" s="5" t="n">
-        <v>2023</v>
+        <v>2026</v>
       </c>
       <c r="D887" s="5" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>0:29:44</t>
         </is>
       </c>
       <c r="E887" s="5" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>0:35:28</t>
         </is>
       </c>
     </row>
@@ -22674,7 +22674,7 @@
         </is>
       </c>
       <c r="C888" s="9" t="n">
-        <v>2024</v>
+        <v>2023</v>
       </c>
       <c r="D888" s="9" t="inlineStr">
         <is>
@@ -22699,7 +22699,7 @@
         </is>
       </c>
       <c r="C889" s="5" t="n">
-        <v>2025</v>
+        <v>2024</v>
       </c>
       <c r="D889" s="5" t="inlineStr">
         <is>
@@ -22724,7 +22724,7 @@
         </is>
       </c>
       <c r="C890" s="9" t="n">
-        <v>2026</v>
+        <v>2025</v>
       </c>
       <c r="D890" s="9" t="inlineStr">
         <is>
@@ -22740,7 +22740,7 @@
     <row r="891">
       <c r="A891" s="4" t="inlineStr">
         <is>
-          <t>Great Scottish Run 10K</t>
+          <t>EDP Meia Maratona de Lisboa - Vodafone 10K</t>
         </is>
       </c>
       <c r="B891" s="5" t="inlineStr">
@@ -22749,7 +22749,7 @@
         </is>
       </c>
       <c r="C891" s="5" t="n">
-        <v>2025</v>
+        <v>2026</v>
       </c>
       <c r="D891" s="5" t="inlineStr">
         <is>
@@ -22765,7 +22765,7 @@
     <row r="892">
       <c r="A892" s="8" t="inlineStr">
         <is>
-          <t>NN CPC Loop Den Haag - 10 KM Loop</t>
+          <t>Great Scottish Run 10K</t>
         </is>
       </c>
       <c r="B892" s="9" t="inlineStr">
@@ -22774,7 +22774,7 @@
         </is>
       </c>
       <c r="C892" s="9" t="n">
-        <v>2026</v>
+        <v>2025</v>
       </c>
       <c r="D892" s="9" t="inlineStr">
         <is>
@@ -22790,7 +22790,7 @@
     <row r="893">
       <c r="A893" s="4" t="inlineStr">
         <is>
-          <t>NN San Silvestre Vallecana</t>
+          <t>NN CPC Loop Den Haag - 10 KM Loop</t>
         </is>
       </c>
       <c r="B893" s="5" t="inlineStr">
@@ -22799,7 +22799,7 @@
         </is>
       </c>
       <c r="C893" s="5" t="n">
-        <v>2023</v>
+        <v>2026</v>
       </c>
       <c r="D893" s="5" t="inlineStr">
         <is>
@@ -22824,7 +22824,7 @@
         </is>
       </c>
       <c r="C894" s="9" t="n">
-        <v>2024</v>
+        <v>2023</v>
       </c>
       <c r="D894" s="9" t="inlineStr">
         <is>
@@ -22833,7 +22833,7 @@
       </c>
       <c r="E894" s="9" t="inlineStr">
         <is>
-          <t>0:31:18</t>
+          <t>N/A</t>
         </is>
       </c>
     </row>
@@ -22849,23 +22849,23 @@
         </is>
       </c>
       <c r="C895" s="5" t="n">
-        <v>2025</v>
+        <v>2024</v>
       </c>
       <c r="D895" s="5" t="inlineStr">
         <is>
-          <t>0:27:41</t>
+          <t>N/A</t>
         </is>
       </c>
       <c r="E895" s="5" t="inlineStr">
         <is>
-          <t>0:31:11</t>
+          <t>0:31:18</t>
         </is>
       </c>
     </row>
     <row r="896">
       <c r="A896" s="8" t="inlineStr">
         <is>
-          <t>Royal Run</t>
+          <t>NN San Silvestre Vallecana</t>
         </is>
       </c>
       <c r="B896" s="9" t="inlineStr">
@@ -22874,16 +22874,16 @@
         </is>
       </c>
       <c r="C896" s="9" t="n">
-        <v>2023</v>
+        <v>2025</v>
       </c>
       <c r="D896" s="9" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>0:27:41</t>
         </is>
       </c>
       <c r="E896" s="9" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>0:31:11</t>
         </is>
       </c>
     </row>
@@ -22899,7 +22899,7 @@
         </is>
       </c>
       <c r="C897" s="5" t="n">
-        <v>2024</v>
+        <v>2023</v>
       </c>
       <c r="D897" s="5" t="inlineStr">
         <is>
@@ -22924,7 +22924,7 @@
         </is>
       </c>
       <c r="C898" s="9" t="n">
-        <v>2025</v>
+        <v>2024</v>
       </c>
       <c r="D898" s="9" t="inlineStr">
         <is>
@@ -22940,7 +22940,7 @@
     <row r="899">
       <c r="A899" s="4" t="inlineStr">
         <is>
-          <t>Run in Lyon</t>
+          <t>Royal Run</t>
         </is>
       </c>
       <c r="B899" s="5" t="inlineStr">
@@ -22965,7 +22965,7 @@
     <row r="900">
       <c r="A900" s="8" t="inlineStr">
         <is>
-          <t>Run in Lyon (10K)</t>
+          <t>Run in Lyon</t>
         </is>
       </c>
       <c r="B900" s="9" t="inlineStr">
@@ -22974,7 +22974,7 @@
         </is>
       </c>
       <c r="C900" s="9" t="n">
-        <v>2023</v>
+        <v>2025</v>
       </c>
       <c r="D900" s="9" t="inlineStr">
         <is>
@@ -22999,7 +22999,7 @@
         </is>
       </c>
       <c r="C901" s="5" t="n">
-        <v>2024</v>
+        <v>2023</v>
       </c>
       <c r="D901" s="5" t="inlineStr">
         <is>
@@ -23024,7 +23024,7 @@
         </is>
       </c>
       <c r="C902" s="9" t="n">
-        <v>2025</v>
+        <v>2024</v>
       </c>
       <c r="D902" s="9" t="inlineStr">
         <is>
@@ -23040,7 +23040,7 @@
     <row r="903">
       <c r="A903" s="4" t="inlineStr">
         <is>
-          <t>Saucony London 10K</t>
+          <t>Run in Lyon (10K)</t>
         </is>
       </c>
       <c r="B903" s="5" t="inlineStr">
@@ -23049,7 +23049,7 @@
         </is>
       </c>
       <c r="C903" s="5" t="n">
-        <v>2023</v>
+        <v>2025</v>
       </c>
       <c r="D903" s="5" t="inlineStr">
         <is>
@@ -23074,16 +23074,16 @@
         </is>
       </c>
       <c r="C904" s="9" t="n">
-        <v>2024</v>
+        <v>2023</v>
       </c>
       <c r="D904" s="9" t="inlineStr">
         <is>
-          <t>0:29:41</t>
+          <t>N/A</t>
         </is>
       </c>
       <c r="E904" s="9" t="inlineStr">
         <is>
-          <t>0:32:51</t>
+          <t>N/A</t>
         </is>
       </c>
     </row>
@@ -23099,16 +23099,16 @@
         </is>
       </c>
       <c r="C905" s="5" t="n">
-        <v>2025</v>
+        <v>2024</v>
       </c>
       <c r="D905" s="5" t="inlineStr">
         <is>
-          <t>0:29:33</t>
+          <t>0:29:41</t>
         </is>
       </c>
       <c r="E905" s="5" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>0:32:51</t>
         </is>
       </c>
     </row>
@@ -23124,23 +23124,23 @@
         </is>
       </c>
       <c r="C906" s="9" t="n">
-        <v>2026</v>
+        <v>2025</v>
       </c>
       <c r="D906" s="9" t="inlineStr">
         <is>
-          <t>0:29:48</t>
+          <t>0:29:33</t>
         </is>
       </c>
       <c r="E906" s="9" t="inlineStr">
         <is>
-          <t>0:33:50</t>
+          <t>N/A</t>
         </is>
       </c>
     </row>
     <row r="907">
       <c r="A907" s="4" t="inlineStr">
         <is>
-          <t>Standard Chartered KL 10K</t>
+          <t>Saucony London 10K</t>
         </is>
       </c>
       <c r="B907" s="5" t="inlineStr">
@@ -23149,23 +23149,23 @@
         </is>
       </c>
       <c r="C907" s="5" t="n">
-        <v>2025</v>
+        <v>2026</v>
       </c>
       <c r="D907" s="5" t="inlineStr">
         <is>
-          <t>0:32:26</t>
+          <t>0:29:48</t>
         </is>
       </c>
       <c r="E907" s="5" t="inlineStr">
         <is>
-          <t>0:39:23</t>
+          <t>0:33:50</t>
         </is>
       </c>
     </row>
     <row r="908">
       <c r="A908" s="8" t="inlineStr">
         <is>
-          <t>Statesman Capitol 10K</t>
+          <t>Standard Chartered KL 10K</t>
         </is>
       </c>
       <c r="B908" s="9" t="inlineStr">
@@ -23174,16 +23174,16 @@
         </is>
       </c>
       <c r="C908" s="9" t="n">
-        <v>2023</v>
+        <v>2025</v>
       </c>
       <c r="D908" s="9" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>0:32:26</t>
         </is>
       </c>
       <c r="E908" s="9" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>0:39:23</t>
         </is>
       </c>
     </row>
@@ -23199,7 +23199,7 @@
         </is>
       </c>
       <c r="C909" s="5" t="n">
-        <v>2024</v>
+        <v>2023</v>
       </c>
       <c r="D909" s="5" t="inlineStr">
         <is>
@@ -23224,7 +23224,7 @@
         </is>
       </c>
       <c r="C910" s="9" t="n">
-        <v>2025</v>
+        <v>2024</v>
       </c>
       <c r="D910" s="9" t="inlineStr">
         <is>
@@ -23240,7 +23240,7 @@
     <row r="911">
       <c r="A911" s="4" t="inlineStr">
         <is>
-          <t>Transurban Bridge to Brisbane</t>
+          <t>Statesman Capitol 10K</t>
         </is>
       </c>
       <c r="B911" s="5" t="inlineStr">
@@ -23249,7 +23249,7 @@
         </is>
       </c>
       <c r="C911" s="5" t="n">
-        <v>2023</v>
+        <v>2025</v>
       </c>
       <c r="D911" s="5" t="inlineStr">
         <is>
@@ -23274,7 +23274,7 @@
         </is>
       </c>
       <c r="C912" s="9" t="n">
-        <v>2024</v>
+        <v>2023</v>
       </c>
       <c r="D912" s="9" t="inlineStr">
         <is>
@@ -23299,7 +23299,7 @@
         </is>
       </c>
       <c r="C913" s="5" t="n">
-        <v>2025</v>
+        <v>2024</v>
       </c>
       <c r="D913" s="5" t="inlineStr">
         <is>
@@ -23315,7 +23315,7 @@
     <row r="914">
       <c r="A914" s="8" t="inlineStr">
         <is>
-          <t>Ukrop's Monument Avenue 10K</t>
+          <t>Transurban Bridge to Brisbane</t>
         </is>
       </c>
       <c r="B914" s="9" t="inlineStr">
@@ -23324,7 +23324,7 @@
         </is>
       </c>
       <c r="C914" s="9" t="n">
-        <v>2023</v>
+        <v>2025</v>
       </c>
       <c r="D914" s="9" t="inlineStr">
         <is>
@@ -23349,7 +23349,7 @@
         </is>
       </c>
       <c r="C915" s="5" t="n">
-        <v>2024</v>
+        <v>2023</v>
       </c>
       <c r="D915" s="5" t="inlineStr">
         <is>
@@ -23374,7 +23374,7 @@
         </is>
       </c>
       <c r="C916" s="9" t="n">
-        <v>2025</v>
+        <v>2024</v>
       </c>
       <c r="D916" s="9" t="inlineStr">
         <is>
@@ -23399,23 +23399,23 @@
         </is>
       </c>
       <c r="C917" s="5" t="n">
-        <v>2026</v>
+        <v>2025</v>
       </c>
       <c r="D917" s="5" t="inlineStr">
         <is>
-          <t>0:30:04</t>
+          <t>N/A</t>
         </is>
       </c>
       <c r="E917" s="5" t="inlineStr">
         <is>
-          <t>0:33:54</t>
+          <t>N/A</t>
         </is>
       </c>
     </row>
     <row r="918">
       <c r="A918" s="8" t="inlineStr">
         <is>
-          <t>VHI Women's Mini Marathon</t>
+          <t>Ukrop's Monument Avenue 10K</t>
         </is>
       </c>
       <c r="B918" s="9" t="inlineStr">
@@ -23428,19 +23428,19 @@
       </c>
       <c r="D918" s="9" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>0:30:04</t>
         </is>
       </c>
       <c r="E918" s="9" t="inlineStr">
         <is>
-          <t>0:31:41</t>
+          <t>0:33:54</t>
         </is>
       </c>
     </row>
     <row r="919">
       <c r="A919" s="4" t="inlineStr">
         <is>
-          <t>Vancouver Sun Run</t>
+          <t>VHI Women's Mini Marathon</t>
         </is>
       </c>
       <c r="B919" s="5" t="inlineStr">
@@ -23449,7 +23449,7 @@
         </is>
       </c>
       <c r="C919" s="5" t="n">
-        <v>2023</v>
+        <v>2026</v>
       </c>
       <c r="D919" s="5" t="inlineStr">
         <is>
@@ -23458,7 +23458,7 @@
       </c>
       <c r="E919" s="5" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>0:31:41</t>
         </is>
       </c>
     </row>
@@ -23474,7 +23474,7 @@
         </is>
       </c>
       <c r="C920" s="9" t="n">
-        <v>2024</v>
+        <v>2023</v>
       </c>
       <c r="D920" s="9" t="inlineStr">
         <is>
@@ -23499,23 +23499,23 @@
         </is>
       </c>
       <c r="C921" s="5" t="n">
-        <v>2025</v>
+        <v>2024</v>
       </c>
       <c r="D921" s="5" t="inlineStr">
         <is>
-          <t>0:28:09</t>
+          <t>N/A</t>
         </is>
       </c>
       <c r="E921" s="5" t="inlineStr">
         <is>
-          <t>0:32:54</t>
+          <t>N/A</t>
         </is>
       </c>
     </row>
     <row r="922">
       <c r="A922" s="8" t="inlineStr">
         <is>
-          <t>Vitality London 10,000</t>
+          <t>Vancouver Sun Run</t>
         </is>
       </c>
       <c r="B922" s="9" t="inlineStr">
@@ -23524,16 +23524,16 @@
         </is>
       </c>
       <c r="C922" s="9" t="n">
-        <v>2023</v>
+        <v>2025</v>
       </c>
       <c r="D922" s="9" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>0:28:09</t>
         </is>
       </c>
       <c r="E922" s="9" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>0:32:54</t>
         </is>
       </c>
     </row>
@@ -23549,16 +23549,16 @@
         </is>
       </c>
       <c r="C923" s="5" t="n">
-        <v>2024</v>
+        <v>2023</v>
       </c>
       <c r="D923" s="5" t="inlineStr">
         <is>
-          <t>0:29:14</t>
+          <t>N/A</t>
         </is>
       </c>
       <c r="E923" s="5" t="inlineStr">
         <is>
-          <t>0:31:36</t>
+          <t>N/A</t>
         </is>
       </c>
     </row>
@@ -23574,23 +23574,23 @@
         </is>
       </c>
       <c r="C924" s="9" t="n">
-        <v>2025</v>
+        <v>2024</v>
       </c>
       <c r="D924" s="9" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>0:29:14</t>
         </is>
       </c>
       <c r="E924" s="9" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>0:31:36</t>
         </is>
       </c>
     </row>
     <row r="925">
       <c r="A925" s="4" t="inlineStr">
         <is>
-          <t>World 10K bengaluru</t>
+          <t>Vitality London 10,000</t>
         </is>
       </c>
       <c r="B925" s="5" t="inlineStr">
@@ -23599,11 +23599,11 @@
         </is>
       </c>
       <c r="C925" s="5" t="n">
-        <v>2026</v>
+        <v>2025</v>
       </c>
       <c r="D925" s="5" t="inlineStr">
         <is>
-          <t>0:27:29</t>
+          <t>N/A</t>
         </is>
       </c>
       <c r="E925" s="5" t="inlineStr">
@@ -23615,20 +23615,20 @@
     <row r="926">
       <c r="A926" s="8" t="inlineStr">
         <is>
-          <t>20KM de Bruxelles</t>
+          <t>World 10K bengaluru</t>
         </is>
       </c>
       <c r="B926" s="9" t="inlineStr">
         <is>
-          <t>AUTRE</t>
+          <t>10K</t>
         </is>
       </c>
       <c r="C926" s="9" t="n">
-        <v>2013</v>
+        <v>2026</v>
       </c>
       <c r="D926" s="9" t="inlineStr">
         <is>
-          <t>0:59:21</t>
+          <t>0:27:29</t>
         </is>
       </c>
       <c r="E926" s="9" t="inlineStr">
@@ -23649,11 +23649,11 @@
         </is>
       </c>
       <c r="C927" s="5" t="n">
-        <v>2014</v>
+        <v>2013</v>
       </c>
       <c r="D927" s="5" t="inlineStr">
         <is>
-          <t>0:59:05</t>
+          <t>0:59:21</t>
         </is>
       </c>
       <c r="E927" s="5" t="inlineStr">
@@ -23674,11 +23674,11 @@
         </is>
       </c>
       <c r="C928" s="9" t="n">
-        <v>2015</v>
+        <v>2014</v>
       </c>
       <c r="D928" s="9" t="inlineStr">
         <is>
-          <t>1:01:47</t>
+          <t>0:59:05</t>
         </is>
       </c>
       <c r="E928" s="9" t="inlineStr">
@@ -23699,16 +23699,16 @@
         </is>
       </c>
       <c r="C929" s="5" t="n">
-        <v>2016</v>
+        <v>2015</v>
       </c>
       <c r="D929" s="5" t="inlineStr">
         <is>
-          <t>1:02:07</t>
+          <t>1:01:47</t>
         </is>
       </c>
       <c r="E929" s="5" t="inlineStr">
         <is>
-          <t>1:13:51</t>
+          <t>N/A</t>
         </is>
       </c>
     </row>
@@ -23724,16 +23724,16 @@
         </is>
       </c>
       <c r="C930" s="9" t="n">
-        <v>2017</v>
+        <v>2016</v>
       </c>
       <c r="D930" s="9" t="inlineStr">
         <is>
-          <t>1:00:37</t>
+          <t>1:02:07</t>
         </is>
       </c>
       <c r="E930" s="9" t="inlineStr">
         <is>
-          <t>1:13:42</t>
+          <t>1:13:51</t>
         </is>
       </c>
     </row>
@@ -23749,16 +23749,16 @@
         </is>
       </c>
       <c r="C931" s="5" t="n">
-        <v>2018</v>
+        <v>2017</v>
       </c>
       <c r="D931" s="5" t="inlineStr">
         <is>
-          <t>1:02:56</t>
+          <t>1:00:37</t>
         </is>
       </c>
       <c r="E931" s="5" t="inlineStr">
         <is>
-          <t>1:14:38</t>
+          <t>1:13:42</t>
         </is>
       </c>
     </row>
@@ -23774,16 +23774,16 @@
         </is>
       </c>
       <c r="C932" s="9" t="n">
-        <v>2019</v>
+        <v>2018</v>
       </c>
       <c r="D932" s="9" t="inlineStr">
         <is>
-          <t>1:00:34</t>
+          <t>1:02:56</t>
         </is>
       </c>
       <c r="E932" s="9" t="inlineStr">
         <is>
-          <t>1:13:04</t>
+          <t>1:14:38</t>
         </is>
       </c>
     </row>
@@ -23799,16 +23799,16 @@
         </is>
       </c>
       <c r="C933" s="5" t="n">
-        <v>2021</v>
+        <v>2019</v>
       </c>
       <c r="D933" s="5" t="inlineStr">
         <is>
-          <t>0:59:31</t>
+          <t>1:00:34</t>
         </is>
       </c>
       <c r="E933" s="5" t="inlineStr">
         <is>
-          <t>1:09:50</t>
+          <t>1:13:04</t>
         </is>
       </c>
     </row>
@@ -23824,16 +23824,16 @@
         </is>
       </c>
       <c r="C934" s="9" t="n">
-        <v>2022</v>
+        <v>2021</v>
       </c>
       <c r="D934" s="9" t="inlineStr">
         <is>
-          <t>1:00:01</t>
+          <t>0:59:31</t>
         </is>
       </c>
       <c r="E934" s="9" t="inlineStr">
         <is>
-          <t>1:11:11</t>
+          <t>1:09:50</t>
         </is>
       </c>
     </row>
@@ -23849,16 +23849,16 @@
         </is>
       </c>
       <c r="C935" s="5" t="n">
-        <v>2023</v>
+        <v>2022</v>
       </c>
       <c r="D935" s="5" t="inlineStr">
         <is>
-          <t>1:00:15</t>
+          <t>1:00:01</t>
         </is>
       </c>
       <c r="E935" s="5" t="inlineStr">
         <is>
-          <t>1:10:44</t>
+          <t>1:11:11</t>
         </is>
       </c>
     </row>
@@ -23874,16 +23874,16 @@
         </is>
       </c>
       <c r="C936" s="9" t="n">
-        <v>2024</v>
+        <v>2023</v>
       </c>
       <c r="D936" s="9" t="inlineStr">
         <is>
-          <t>0:59:57</t>
+          <t>1:00:15</t>
         </is>
       </c>
       <c r="E936" s="9" t="inlineStr">
         <is>
-          <t>1:10:56</t>
+          <t>1:10:44</t>
         </is>
       </c>
     </row>
@@ -23899,16 +23899,16 @@
         </is>
       </c>
       <c r="C937" s="5" t="n">
-        <v>2025</v>
+        <v>2024</v>
       </c>
       <c r="D937" s="5" t="inlineStr">
         <is>
-          <t>0:59:26</t>
+          <t>0:59:57</t>
         </is>
       </c>
       <c r="E937" s="5" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>1:10:56</t>
         </is>
       </c>
     </row>
@@ -23924,66 +23924,66 @@
         </is>
       </c>
       <c r="C938" s="9" t="n">
-        <v>2026</v>
+        <v>2025</v>
       </c>
       <c r="D938" s="9" t="inlineStr">
         <is>
-          <t>0:59:47</t>
+          <t>0:59:26</t>
         </is>
       </c>
       <c r="E938" s="9" t="inlineStr">
         <is>
-          <t>1:11:20</t>
+          <t>N/A</t>
         </is>
       </c>
     </row>
     <row r="939">
       <c r="A939" s="4" t="inlineStr">
         <is>
-          <t>AJ Bell Great Birmingham Run</t>
+          <t>20KM de Bruxelles</t>
         </is>
       </c>
       <c r="B939" s="5" t="inlineStr">
         <is>
-          <t>SEMI</t>
+          <t>AUTRE</t>
         </is>
       </c>
       <c r="C939" s="5" t="n">
-        <v>2025</v>
+        <v>2026</v>
       </c>
       <c r="D939" s="5" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>0:59:47</t>
         </is>
       </c>
       <c r="E939" s="5" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>1:11:20</t>
         </is>
       </c>
     </row>
     <row r="940">
       <c r="A940" s="8" t="inlineStr">
         <is>
-          <t>AJ Bell Great South Run</t>
+          <t>AJ Bell Great Birmingham Run</t>
         </is>
       </c>
       <c r="B940" s="9" t="inlineStr">
         <is>
-          <t>AUTRE</t>
+          <t>SEMI</t>
         </is>
       </c>
       <c r="C940" s="9" t="n">
-        <v>2021</v>
+        <v>2025</v>
       </c>
       <c r="D940" s="9" t="inlineStr">
         <is>
-          <t>0:47:19</t>
+          <t>N/A</t>
         </is>
       </c>
       <c r="E940" s="9" t="inlineStr">
         <is>
-          <t>0:50:42</t>
+          <t>N/A</t>
         </is>
       </c>
     </row>
@@ -23999,23 +23999,23 @@
         </is>
       </c>
       <c r="C941" s="5" t="n">
-        <v>2025</v>
+        <v>2021</v>
       </c>
       <c r="D941" s="5" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>0:47:19</t>
         </is>
       </c>
       <c r="E941" s="5" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>0:50:42</t>
         </is>
       </c>
     </row>
     <row r="942">
       <c r="A942" s="8" t="inlineStr">
         <is>
-          <t>Army Ten Miler</t>
+          <t>AJ Bell Great South Run</t>
         </is>
       </c>
       <c r="B942" s="9" t="inlineStr">
@@ -24040,7 +24040,7 @@
     <row r="943">
       <c r="A943" s="4" t="inlineStr">
         <is>
-          <t>Baloise Antwerp 10 miles</t>
+          <t>Army Ten Miler</t>
         </is>
       </c>
       <c r="B943" s="5" t="inlineStr">
@@ -24049,11 +24049,11 @@
         </is>
       </c>
       <c r="C943" s="5" t="n">
-        <v>2022</v>
+        <v>2025</v>
       </c>
       <c r="D943" s="5" t="inlineStr">
         <is>
-          <t>0:48:48</t>
+          <t>N/A</t>
         </is>
       </c>
       <c r="E943" s="5" t="inlineStr">
@@ -24074,11 +24074,11 @@
         </is>
       </c>
       <c r="C944" s="9" t="n">
-        <v>2023</v>
+        <v>2022</v>
       </c>
       <c r="D944" s="9" t="inlineStr">
         <is>
-          <t>0:47:50</t>
+          <t>0:48:48</t>
         </is>
       </c>
       <c r="E944" s="9" t="inlineStr">
@@ -24099,11 +24099,11 @@
         </is>
       </c>
       <c r="C945" s="5" t="n">
-        <v>2024</v>
+        <v>2023</v>
       </c>
       <c r="D945" s="5" t="inlineStr">
         <is>
-          <t>0:47:21</t>
+          <t>0:47:50</t>
         </is>
       </c>
       <c r="E945" s="5" t="inlineStr">
@@ -24115,7 +24115,7 @@
     <row r="946">
       <c r="A946" s="8" t="inlineStr">
         <is>
-          <t>Bay to Breakers</t>
+          <t>Baloise Antwerp 10 miles</t>
         </is>
       </c>
       <c r="B946" s="9" t="inlineStr">
@@ -24124,16 +24124,16 @@
         </is>
       </c>
       <c r="C946" s="9" t="n">
-        <v>2005</v>
+        <v>2024</v>
       </c>
       <c r="D946" s="9" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>0:47:21</t>
         </is>
       </c>
       <c r="E946" s="9" t="inlineStr">
         <is>
-          <t>0:38:22</t>
+          <t>N/A</t>
         </is>
       </c>
     </row>
@@ -24149,16 +24149,16 @@
         </is>
       </c>
       <c r="C947" s="5" t="n">
-        <v>2009</v>
+        <v>2005</v>
       </c>
       <c r="D947" s="5" t="inlineStr">
         <is>
-          <t>0:33:31</t>
+          <t>N/A</t>
         </is>
       </c>
       <c r="E947" s="5" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>0:38:22</t>
         </is>
       </c>
     </row>
@@ -24174,16 +24174,16 @@
         </is>
       </c>
       <c r="C948" s="9" t="n">
-        <v>2010</v>
+        <v>2009</v>
       </c>
       <c r="D948" s="9" t="inlineStr">
         <is>
-          <t>0:34:15</t>
+          <t>0:33:31</t>
         </is>
       </c>
       <c r="E948" s="9" t="inlineStr">
         <is>
-          <t>0:38:07</t>
+          <t>N/A</t>
         </is>
       </c>
     </row>
@@ -24199,16 +24199,16 @@
         </is>
       </c>
       <c r="C949" s="5" t="n">
-        <v>2012</v>
+        <v>2010</v>
       </c>
       <c r="D949" s="5" t="inlineStr">
         <is>
-          <t>0:34:40</t>
+          <t>0:34:15</t>
         </is>
       </c>
       <c r="E949" s="5" t="inlineStr">
         <is>
-          <t>0:39:02</t>
+          <t>0:38:07</t>
         </is>
       </c>
     </row>
@@ -24224,16 +24224,16 @@
         </is>
       </c>
       <c r="C950" s="9" t="n">
-        <v>2019</v>
+        <v>2012</v>
       </c>
       <c r="D950" s="9" t="inlineStr">
         <is>
-          <t>0:35:01</t>
+          <t>0:34:40</t>
         </is>
       </c>
       <c r="E950" s="9" t="inlineStr">
         <is>
-          <t>0:39:28</t>
+          <t>0:39:02</t>
         </is>
       </c>
     </row>
@@ -24249,16 +24249,16 @@
         </is>
       </c>
       <c r="C951" s="5" t="n">
-        <v>2022</v>
+        <v>2019</v>
       </c>
       <c r="D951" s="5" t="inlineStr">
         <is>
-          <t>0:36:10</t>
+          <t>0:35:01</t>
         </is>
       </c>
       <c r="E951" s="5" t="inlineStr">
         <is>
-          <t>0:42:05</t>
+          <t>0:39:28</t>
         </is>
       </c>
     </row>
@@ -24274,23 +24274,23 @@
         </is>
       </c>
       <c r="C952" s="9" t="n">
-        <v>2024</v>
+        <v>2022</v>
       </c>
       <c r="D952" s="9" t="inlineStr">
         <is>
-          <t>0:37:02</t>
+          <t>0:36:10</t>
         </is>
       </c>
       <c r="E952" s="9" t="inlineStr">
         <is>
-          <t>0:43:48</t>
+          <t>0:42:05</t>
         </is>
       </c>
     </row>
     <row r="953">
       <c r="A953" s="4" t="inlineStr">
         <is>
-          <t>Boilermaker Road Race</t>
+          <t>Bay to Breakers</t>
         </is>
       </c>
       <c r="B953" s="5" t="inlineStr">
@@ -24299,23 +24299,23 @@
         </is>
       </c>
       <c r="C953" s="5" t="n">
-        <v>2025</v>
+        <v>2024</v>
       </c>
       <c r="D953" s="5" t="inlineStr">
         <is>
-          <t>0:42:44</t>
+          <t>0:37:02</t>
         </is>
       </c>
       <c r="E953" s="5" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>0:43:48</t>
         </is>
       </c>
     </row>
     <row r="954">
       <c r="A954" s="8" t="inlineStr">
         <is>
-          <t>Broad Street Run</t>
+          <t>Boilermaker Road Race</t>
         </is>
       </c>
       <c r="B954" s="9" t="inlineStr">
@@ -24328,19 +24328,19 @@
       </c>
       <c r="D954" s="9" t="inlineStr">
         <is>
-          <t>0:46:13</t>
+          <t>0:42:44</t>
         </is>
       </c>
       <c r="E954" s="9" t="inlineStr">
         <is>
-          <t>0:54:01</t>
+          <t>N/A</t>
         </is>
       </c>
     </row>
     <row r="955">
       <c r="A955" s="4" t="inlineStr">
         <is>
-          <t>City2Surf</t>
+          <t>Broad Street Run</t>
         </is>
       </c>
       <c r="B955" s="5" t="inlineStr">
@@ -24349,16 +24349,16 @@
         </is>
       </c>
       <c r="C955" s="5" t="n">
-        <v>2024</v>
+        <v>2025</v>
       </c>
       <c r="D955" s="5" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>0:46:13</t>
         </is>
       </c>
       <c r="E955" s="5" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>0:54:01</t>
         </is>
       </c>
     </row>
@@ -24374,23 +24374,23 @@
         </is>
       </c>
       <c r="C956" s="9" t="n">
-        <v>2026</v>
+        <v>2024</v>
       </c>
       <c r="D956" s="9" t="inlineStr">
         <is>
-          <t>0:40:27</t>
+          <t>N/A</t>
         </is>
       </c>
       <c r="E956" s="9" t="inlineStr">
         <is>
-          <t>0:46:35</t>
+          <t>N/A</t>
         </is>
       </c>
     </row>
     <row r="957">
       <c r="A957" s="4" t="inlineStr">
         <is>
-          <t>Dam tot Damloop</t>
+          <t>City2Surf</t>
         </is>
       </c>
       <c r="B957" s="5" t="inlineStr">
@@ -24399,16 +24399,16 @@
         </is>
       </c>
       <c r="C957" s="5" t="n">
-        <v>2009</v>
+        <v>2026</v>
       </c>
       <c r="D957" s="5" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>0:40:27</t>
         </is>
       </c>
       <c r="E957" s="5" t="inlineStr">
         <is>
-          <t>0:50:39</t>
+          <t>0:46:35</t>
         </is>
       </c>
     </row>
@@ -24424,7 +24424,7 @@
         </is>
       </c>
       <c r="C958" s="9" t="n">
-        <v>2010</v>
+        <v>2009</v>
       </c>
       <c r="D958" s="9" t="inlineStr">
         <is>
@@ -24433,7 +24433,7 @@
       </c>
       <c r="E958" s="9" t="inlineStr">
         <is>
-          <t>0:51:30</t>
+          <t>0:50:39</t>
         </is>
       </c>
     </row>
@@ -24449,16 +24449,16 @@
         </is>
       </c>
       <c r="C959" s="5" t="n">
-        <v>2011</v>
+        <v>2010</v>
       </c>
       <c r="D959" s="5" t="inlineStr">
         <is>
-          <t>0:44:27</t>
+          <t>N/A</t>
         </is>
       </c>
       <c r="E959" s="5" t="inlineStr">
         <is>
-          <t>0:51:57</t>
+          <t>0:51:30</t>
         </is>
       </c>
     </row>
@@ -24474,16 +24474,16 @@
         </is>
       </c>
       <c r="C960" s="9" t="n">
-        <v>2012</v>
+        <v>2011</v>
       </c>
       <c r="D960" s="9" t="inlineStr">
         <is>
-          <t>0:44:48</t>
+          <t>0:44:27</t>
         </is>
       </c>
       <c r="E960" s="9" t="inlineStr">
         <is>
-          <t>0:51:42</t>
+          <t>0:51:57</t>
         </is>
       </c>
     </row>
@@ -24499,16 +24499,16 @@
         </is>
       </c>
       <c r="C961" s="5" t="n">
-        <v>2013</v>
+        <v>2012</v>
       </c>
       <c r="D961" s="5" t="inlineStr">
         <is>
-          <t>0:45:28</t>
+          <t>0:44:48</t>
         </is>
       </c>
       <c r="E961" s="5" t="inlineStr">
         <is>
-          <t>0:51:33</t>
+          <t>0:51:42</t>
         </is>
       </c>
     </row>
@@ -24524,16 +24524,16 @@
         </is>
       </c>
       <c r="C962" s="9" t="n">
-        <v>2014</v>
+        <v>2013</v>
       </c>
       <c r="D962" s="9" t="inlineStr">
         <is>
-          <t>0:45:45</t>
+          <t>0:45:28</t>
         </is>
       </c>
       <c r="E962" s="9" t="inlineStr">
         <is>
-          <t>0:53:09</t>
+          <t>0:51:33</t>
         </is>
       </c>
     </row>
@@ -24549,16 +24549,16 @@
         </is>
       </c>
       <c r="C963" s="5" t="n">
-        <v>2019</v>
+        <v>2014</v>
       </c>
       <c r="D963" s="5" t="inlineStr">
         <is>
-          <t>0:45:15</t>
+          <t>0:45:45</t>
         </is>
       </c>
       <c r="E963" s="5" t="inlineStr">
         <is>
-          <t>0:50:45</t>
+          <t>0:53:09</t>
         </is>
       </c>
     </row>
@@ -24574,16 +24574,16 @@
         </is>
       </c>
       <c r="C964" s="9" t="n">
-        <v>2022</v>
+        <v>2019</v>
       </c>
       <c r="D964" s="9" t="inlineStr">
         <is>
-          <t>0:49:00</t>
+          <t>0:45:15</t>
         </is>
       </c>
       <c r="E964" s="9" t="inlineStr">
         <is>
-          <t>0:55:44</t>
+          <t>0:50:45</t>
         </is>
       </c>
     </row>
@@ -24599,16 +24599,16 @@
         </is>
       </c>
       <c r="C965" s="5" t="n">
-        <v>2024</v>
+        <v>2022</v>
       </c>
       <c r="D965" s="5" t="inlineStr">
         <is>
-          <t>0:44:51</t>
+          <t>0:49:00</t>
         </is>
       </c>
       <c r="E965" s="5" t="inlineStr">
         <is>
-          <t>0:51:15</t>
+          <t>0:55:44</t>
         </is>
       </c>
     </row>
@@ -24624,23 +24624,23 @@
         </is>
       </c>
       <c r="C966" s="9" t="n">
-        <v>2025</v>
+        <v>2024</v>
       </c>
       <c r="D966" s="9" t="inlineStr">
         <is>
-          <t>0:46:07</t>
+          <t>0:44:51</t>
         </is>
       </c>
       <c r="E966" s="9" t="inlineStr">
         <is>
-          <t>0:50:51</t>
+          <t>0:51:15</t>
         </is>
       </c>
     </row>
     <row r="967">
       <c r="A967" s="4" t="inlineStr">
         <is>
-          <t>Falmouth Road Race</t>
+          <t>Dam tot Damloop</t>
         </is>
       </c>
       <c r="B967" s="5" t="inlineStr">
@@ -24653,19 +24653,19 @@
       </c>
       <c r="D967" s="5" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>0:46:07</t>
         </is>
       </c>
       <c r="E967" s="5" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>0:50:51</t>
         </is>
       </c>
     </row>
     <row r="968">
       <c r="A968" s="8" t="inlineStr">
         <is>
-          <t>Grand Prix Von Bern</t>
+          <t>Falmouth Road Race</t>
         </is>
       </c>
       <c r="B968" s="9" t="inlineStr">
@@ -24674,53 +24674,53 @@
         </is>
       </c>
       <c r="C968" s="9" t="n">
-        <v>2026</v>
+        <v>2025</v>
       </c>
       <c r="D968" s="9" t="inlineStr">
         <is>
-          <t>0:46:58</t>
+          <t>N/A</t>
         </is>
       </c>
       <c r="E968" s="9" t="inlineStr">
         <is>
-          <t>0:55:50</t>
+          <t>N/A</t>
         </is>
       </c>
     </row>
     <row r="969">
       <c r="A969" s="4" t="inlineStr">
         <is>
-          <t>Great Scottish Run</t>
+          <t>Grand Prix Von Bern</t>
         </is>
       </c>
       <c r="B969" s="5" t="inlineStr">
         <is>
-          <t>SEMI</t>
+          <t>AUTRE</t>
         </is>
       </c>
       <c r="C969" s="5" t="n">
-        <v>2025</v>
+        <v>2026</v>
       </c>
       <c r="D969" s="5" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>0:46:58</t>
         </is>
       </c>
       <c r="E969" s="5" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>0:55:50</t>
         </is>
       </c>
     </row>
     <row r="970">
       <c r="A970" s="8" t="inlineStr">
         <is>
-          <t>Lilac Bloomsday Run</t>
+          <t>Great Scottish Run</t>
         </is>
       </c>
       <c r="B970" s="9" t="inlineStr">
         <is>
-          <t>AUTRE</t>
+          <t>SEMI</t>
         </is>
       </c>
       <c r="C970" s="9" t="n">
@@ -24740,30 +24740,55 @@
     <row r="971">
       <c r="A971" s="4" t="inlineStr">
         <is>
+          <t>Lilac Bloomsday Run</t>
+        </is>
+      </c>
+      <c r="B971" s="5" t="inlineStr">
+        <is>
+          <t>AUTRE</t>
+        </is>
+      </c>
+      <c r="C971" s="5" t="n">
+        <v>2025</v>
+      </c>
+      <c r="D971" s="5" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="E971" s="5" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+    </row>
+    <row r="972">
+      <c r="A972" s="8" t="inlineStr">
+        <is>
           <t>Manchester Road Race</t>
         </is>
       </c>
-      <c r="B971" s="5" t="inlineStr">
+      <c r="B972" s="9" t="inlineStr">
         <is>
           <t>AUTRE</t>
         </is>
       </c>
-      <c r="C971" s="5" t="n">
+      <c r="C972" s="9" t="n">
         <v>2024</v>
       </c>
-      <c r="D971" s="5" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="E971" s="5" t="inlineStr">
+      <c r="D972" s="9" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="E972" s="9" t="inlineStr">
         <is>
           <t>N/A</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:E971"/>
+  <autoFilter ref="A1:E972"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Auto Update 4D 2026-10-10 — 1 ecriture(s) (11 deja remplie(s))
</commit_message>
<xml_diff>
--- a/Chronos_Vainqueurs.xlsx
+++ b/Chronos_Vainqueurs.xlsx
@@ -10,7 +10,7 @@
     <sheet name="Chronos Vainqueurs" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Chronos Vainqueurs'!$A$1:$E$981</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Chronos Vainqueurs'!$A$1:$E$982</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -475,7 +475,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E981"/>
+  <dimension ref="A1:E982"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="50" customWidth="1" min="1" max="1"/>
@@ -24940,7 +24940,7 @@
     <row r="979">
       <c r="A979" s="4" t="inlineStr">
         <is>
-          <t>Lilac Bloomsday Run</t>
+          <t>Harmonie Mutuelle 20km de Paris</t>
         </is>
       </c>
       <c r="B979" s="5" t="inlineStr">
@@ -24949,23 +24949,23 @@
         </is>
       </c>
       <c r="C979" s="5" t="n">
-        <v>2025</v>
+        <v>2026</v>
       </c>
       <c r="D979" s="5" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>00:57:11</t>
         </is>
       </c>
       <c r="E979" s="5" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>01:04:35</t>
         </is>
       </c>
     </row>
     <row r="980">
       <c r="A980" s="8" t="inlineStr">
         <is>
-          <t>Manchester Road Race</t>
+          <t>Lilac Bloomsday Run</t>
         </is>
       </c>
       <c r="B980" s="9" t="inlineStr">
@@ -24974,7 +24974,7 @@
         </is>
       </c>
       <c r="C980" s="9" t="n">
-        <v>2024</v>
+        <v>2025</v>
       </c>
       <c r="D980" s="9" t="inlineStr">
         <is>
@@ -24990,30 +24990,55 @@
     <row r="981">
       <c r="A981" s="4" t="inlineStr">
         <is>
+          <t>Manchester Road Race</t>
+        </is>
+      </c>
+      <c r="B981" s="5" t="inlineStr">
+        <is>
+          <t>AUTRE</t>
+        </is>
+      </c>
+      <c r="C981" s="5" t="n">
+        <v>2024</v>
+      </c>
+      <c r="D981" s="5" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="E981" s="5" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+    </row>
+    <row r="982">
+      <c r="A982" s="8" t="inlineStr">
+        <is>
           <t>Paris-Versailles - La grande classique</t>
         </is>
       </c>
-      <c r="B981" s="5" t="inlineStr">
+      <c r="B982" s="9" t="inlineStr">
         <is>
           <t>AUTRE</t>
         </is>
       </c>
-      <c r="C981" s="5" t="n">
+      <c r="C982" s="9" t="n">
         <v>2026</v>
       </c>
-      <c r="D981" s="5" t="inlineStr">
+      <c r="D982" s="9" t="inlineStr">
         <is>
           <t>00:49:05</t>
         </is>
       </c>
-      <c r="E981" s="5" t="inlineStr">
+      <c r="E982" s="9" t="inlineStr">
         <is>
           <t>00:55:58</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:E981"/>
+  <autoFilter ref="A1:E982"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Renommer « Nike Half Marathon » en « Nike Melbourne Half Marathon »
Le nom precedent etait le seul du dashboard sans ville, ce qui le rendait
ambigu a cote des autres semis. Renommage propage dans l'Excel (onglet ALL
puis onglets par distance regeneres) et dans les douze fichiers qui le
portaient, dont temp_chronos_1.json et update_log.json ecrits depuis le
renommage precedent.

Verifie apres generation : plus aucune occurrence de l'ancien nom, les deux
lignes de Melbourne portent la bonne distance et leurs chronos.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01NDRDdaoD47bJRT7WbM1up5
</commit_message>
<xml_diff>
--- a/Chronos_Vainqueurs.xlsx
+++ b/Chronos_Vainqueurs.xlsx
@@ -20415,7 +20415,7 @@
     <row r="798">
       <c r="A798" s="6" t="inlineStr">
         <is>
-          <t>Nike Half Marathon</t>
+          <t>Nike Melbourne Half Marathon</t>
         </is>
       </c>
       <c r="B798" s="7" t="inlineStr">
@@ -20440,7 +20440,7 @@
     <row r="799">
       <c r="A799" s="4" t="inlineStr">
         <is>
-          <t>Nike Half Marathon</t>
+          <t>Nike Melbourne Half Marathon</t>
         </is>
       </c>
       <c r="B799" s="5" t="inlineStr">

</xml_diff>

<commit_message>
TCS World 10K Bengaluru : renommage, organisateur, sponsoring
- "World 10K bengaluru" -> "TCS World 10K Bengaluru" (Excel ALL + onglets
  distance, event_countries.json, sponsoring_data.json, create_chronos.py)
- Organisateur : Procam International
- IDFC FIRST Bank : associate -> official (le type associate n'etait rendu
  dans aucun seau de l'onglet Sponsoring)
- TCS deja enregistre partenaire titre 2008-2026, inchange

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01NDRDdaoD47bJRT7WbM1up5
</commit_message>
<xml_diff>
--- a/Chronos_Vainqueurs.xlsx
+++ b/Chronos_Vainqueurs.xlsx
@@ -23615,7 +23615,7 @@
     <row r="926">
       <c r="A926" s="8" t="inlineStr">
         <is>
-          <t>Transurban Bridge to Brisbane</t>
+          <t>TCS World 10K Bengaluru</t>
         </is>
       </c>
       <c r="B926" s="9" t="inlineStr">
@@ -23624,11 +23624,11 @@
         </is>
       </c>
       <c r="C926" s="9" t="n">
-        <v>2023</v>
+        <v>2026</v>
       </c>
       <c r="D926" s="9" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>0:27:29</t>
         </is>
       </c>
       <c r="E926" s="9" t="inlineStr">
@@ -23649,7 +23649,7 @@
         </is>
       </c>
       <c r="C927" s="5" t="n">
-        <v>2024</v>
+        <v>2023</v>
       </c>
       <c r="D927" s="5" t="inlineStr">
         <is>
@@ -23674,7 +23674,7 @@
         </is>
       </c>
       <c r="C928" s="9" t="n">
-        <v>2025</v>
+        <v>2024</v>
       </c>
       <c r="D928" s="9" t="inlineStr">
         <is>
@@ -23690,7 +23690,7 @@
     <row r="929">
       <c r="A929" s="4" t="inlineStr">
         <is>
-          <t>Ukrop's Monument Avenue 10K</t>
+          <t>Transurban Bridge to Brisbane</t>
         </is>
       </c>
       <c r="B929" s="5" t="inlineStr">
@@ -23699,7 +23699,7 @@
         </is>
       </c>
       <c r="C929" s="5" t="n">
-        <v>2023</v>
+        <v>2025</v>
       </c>
       <c r="D929" s="5" t="inlineStr">
         <is>
@@ -23724,7 +23724,7 @@
         </is>
       </c>
       <c r="C930" s="9" t="n">
-        <v>2024</v>
+        <v>2023</v>
       </c>
       <c r="D930" s="9" t="inlineStr">
         <is>
@@ -23749,7 +23749,7 @@
         </is>
       </c>
       <c r="C931" s="5" t="n">
-        <v>2025</v>
+        <v>2024</v>
       </c>
       <c r="D931" s="5" t="inlineStr">
         <is>
@@ -23774,23 +23774,23 @@
         </is>
       </c>
       <c r="C932" s="9" t="n">
-        <v>2026</v>
+        <v>2025</v>
       </c>
       <c r="D932" s="9" t="inlineStr">
         <is>
-          <t>0:30:04</t>
+          <t>N/A</t>
         </is>
       </c>
       <c r="E932" s="9" t="inlineStr">
         <is>
-          <t>0:33:54</t>
+          <t>N/A</t>
         </is>
       </c>
     </row>
     <row r="933">
       <c r="A933" s="4" t="inlineStr">
         <is>
-          <t>VHI Women's Mini Marathon</t>
+          <t>Ukrop's Monument Avenue 10K</t>
         </is>
       </c>
       <c r="B933" s="5" t="inlineStr">
@@ -23803,19 +23803,19 @@
       </c>
       <c r="D933" s="5" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>0:30:04</t>
         </is>
       </c>
       <c r="E933" s="5" t="inlineStr">
         <is>
-          <t>0:31:41</t>
+          <t>0:33:54</t>
         </is>
       </c>
     </row>
     <row r="934">
       <c r="A934" s="8" t="inlineStr">
         <is>
-          <t>Vancouver Sun Run</t>
+          <t>VHI Women's Mini Marathon</t>
         </is>
       </c>
       <c r="B934" s="9" t="inlineStr">
@@ -23824,7 +23824,7 @@
         </is>
       </c>
       <c r="C934" s="9" t="n">
-        <v>2023</v>
+        <v>2026</v>
       </c>
       <c r="D934" s="9" t="inlineStr">
         <is>
@@ -23833,7 +23833,7 @@
       </c>
       <c r="E934" s="9" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>0:31:41</t>
         </is>
       </c>
     </row>
@@ -23849,7 +23849,7 @@
         </is>
       </c>
       <c r="C935" s="5" t="n">
-        <v>2024</v>
+        <v>2023</v>
       </c>
       <c r="D935" s="5" t="inlineStr">
         <is>
@@ -23874,23 +23874,23 @@
         </is>
       </c>
       <c r="C936" s="9" t="n">
-        <v>2025</v>
+        <v>2024</v>
       </c>
       <c r="D936" s="9" t="inlineStr">
         <is>
-          <t>0:28:09</t>
+          <t>N/A</t>
         </is>
       </c>
       <c r="E936" s="9" t="inlineStr">
         <is>
-          <t>0:32:54</t>
+          <t>N/A</t>
         </is>
       </c>
     </row>
     <row r="937">
       <c r="A937" s="4" t="inlineStr">
         <is>
-          <t>Vitality London 10,000</t>
+          <t>Vancouver Sun Run</t>
         </is>
       </c>
       <c r="B937" s="5" t="inlineStr">
@@ -23899,16 +23899,16 @@
         </is>
       </c>
       <c r="C937" s="5" t="n">
-        <v>2023</v>
+        <v>2025</v>
       </c>
       <c r="D937" s="5" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>0:28:09</t>
         </is>
       </c>
       <c r="E937" s="5" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>0:32:54</t>
         </is>
       </c>
     </row>
@@ -23924,16 +23924,16 @@
         </is>
       </c>
       <c r="C938" s="9" t="n">
-        <v>2024</v>
+        <v>2023</v>
       </c>
       <c r="D938" s="9" t="inlineStr">
         <is>
-          <t>0:29:14</t>
+          <t>N/A</t>
         </is>
       </c>
       <c r="E938" s="9" t="inlineStr">
         <is>
-          <t>0:31:36</t>
+          <t>N/A</t>
         </is>
       </c>
     </row>
@@ -23949,23 +23949,23 @@
         </is>
       </c>
       <c r="C939" s="5" t="n">
-        <v>2025</v>
+        <v>2024</v>
       </c>
       <c r="D939" s="5" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>0:29:14</t>
         </is>
       </c>
       <c r="E939" s="5" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>0:31:36</t>
         </is>
       </c>
     </row>
     <row r="940">
       <c r="A940" s="8" t="inlineStr">
         <is>
-          <t>World 10K bengaluru</t>
+          <t>Vitality London 10,000</t>
         </is>
       </c>
       <c r="B940" s="9" t="inlineStr">
@@ -23974,11 +23974,11 @@
         </is>
       </c>
       <c r="C940" s="9" t="n">
-        <v>2026</v>
+        <v>2025</v>
       </c>
       <c r="D940" s="9" t="inlineStr">
         <is>
-          <t>0:27:29</t>
+          <t>N/A</t>
         </is>
       </c>
       <c r="E940" s="9" t="inlineStr">

</xml_diff>

<commit_message>
Baloise Antwerp 10 miles 2026 : Update 4D complet
Source : ChronoRace ctx 20260425_10miles, table LIVE3 (10 miles, 16.09 km,
identifiee par la vitesse du vainqueur). 42 820 lignes parcourues, dont
35 949 avec un temps et la position Finish.

- Finishers : 35949
- Temps moyen : 01:35:23 (moyenne des 35 949 temps nets)
- Vainqueur H : 0:46:43 (Patrick Nimubona)
- Vainqueur F : 0:53:07 (Charlotte Van Hese)

LIVE1 (2 040 inscrits sans temps) et LIVE2 (short run 8 km) ecartees.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01NDRDdaoD47bJRT7WbM1up5
</commit_message>
<xml_diff>
--- a/Chronos_Vainqueurs.xlsx
+++ b/Chronos_Vainqueurs.xlsx
@@ -10,7 +10,7 @@
     <sheet name="Chronos Vainqueurs" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Chronos Vainqueurs'!$A$1:$E$988</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Chronos Vainqueurs'!$A$1:$E$989</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -475,7 +475,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E988"/>
+  <dimension ref="A1:E989"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="50" customWidth="1" min="1" max="1"/>
@@ -24490,7 +24490,7 @@
     <row r="961">
       <c r="A961" s="4" t="inlineStr">
         <is>
-          <t>Bay to Breakers</t>
+          <t>Baloise Antwerp 10 miles</t>
         </is>
       </c>
       <c r="B961" s="5" t="inlineStr">
@@ -24499,16 +24499,16 @@
         </is>
       </c>
       <c r="C961" s="5" t="n">
-        <v>2005</v>
+        <v>2026</v>
       </c>
       <c r="D961" s="5" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>0:46:43</t>
         </is>
       </c>
       <c r="E961" s="5" t="inlineStr">
         <is>
-          <t>0:38:22</t>
+          <t>0:53:07</t>
         </is>
       </c>
     </row>
@@ -24524,16 +24524,16 @@
         </is>
       </c>
       <c r="C962" s="9" t="n">
-        <v>2009</v>
+        <v>2005</v>
       </c>
       <c r="D962" s="9" t="inlineStr">
         <is>
-          <t>0:33:31</t>
+          <t>N/A</t>
         </is>
       </c>
       <c r="E962" s="9" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>0:38:22</t>
         </is>
       </c>
     </row>
@@ -24549,16 +24549,16 @@
         </is>
       </c>
       <c r="C963" s="5" t="n">
-        <v>2010</v>
+        <v>2009</v>
       </c>
       <c r="D963" s="5" t="inlineStr">
         <is>
-          <t>0:34:15</t>
+          <t>0:33:31</t>
         </is>
       </c>
       <c r="E963" s="5" t="inlineStr">
         <is>
-          <t>0:38:07</t>
+          <t>N/A</t>
         </is>
       </c>
     </row>
@@ -24574,16 +24574,16 @@
         </is>
       </c>
       <c r="C964" s="9" t="n">
-        <v>2012</v>
+        <v>2010</v>
       </c>
       <c r="D964" s="9" t="inlineStr">
         <is>
-          <t>0:34:40</t>
+          <t>0:34:15</t>
         </is>
       </c>
       <c r="E964" s="9" t="inlineStr">
         <is>
-          <t>0:39:02</t>
+          <t>0:38:07</t>
         </is>
       </c>
     </row>
@@ -24599,16 +24599,16 @@
         </is>
       </c>
       <c r="C965" s="5" t="n">
-        <v>2019</v>
+        <v>2012</v>
       </c>
       <c r="D965" s="5" t="inlineStr">
         <is>
-          <t>0:35:01</t>
+          <t>0:34:40</t>
         </is>
       </c>
       <c r="E965" s="5" t="inlineStr">
         <is>
-          <t>0:39:28</t>
+          <t>0:39:02</t>
         </is>
       </c>
     </row>
@@ -24624,16 +24624,16 @@
         </is>
       </c>
       <c r="C966" s="9" t="n">
-        <v>2022</v>
+        <v>2019</v>
       </c>
       <c r="D966" s="9" t="inlineStr">
         <is>
-          <t>0:36:10</t>
+          <t>0:35:01</t>
         </is>
       </c>
       <c r="E966" s="9" t="inlineStr">
         <is>
-          <t>0:42:05</t>
+          <t>0:39:28</t>
         </is>
       </c>
     </row>
@@ -24649,23 +24649,23 @@
         </is>
       </c>
       <c r="C967" s="5" t="n">
-        <v>2024</v>
+        <v>2022</v>
       </c>
       <c r="D967" s="5" t="inlineStr">
         <is>
-          <t>0:37:02</t>
+          <t>0:36:10</t>
         </is>
       </c>
       <c r="E967" s="5" t="inlineStr">
         <is>
-          <t>0:43:48</t>
+          <t>0:42:05</t>
         </is>
       </c>
     </row>
     <row r="968">
       <c r="A968" s="8" t="inlineStr">
         <is>
-          <t>Boilermaker Road Race</t>
+          <t>Bay to Breakers</t>
         </is>
       </c>
       <c r="B968" s="9" t="inlineStr">
@@ -24674,23 +24674,23 @@
         </is>
       </c>
       <c r="C968" s="9" t="n">
-        <v>2025</v>
+        <v>2024</v>
       </c>
       <c r="D968" s="9" t="inlineStr">
         <is>
-          <t>0:42:44</t>
+          <t>0:37:02</t>
         </is>
       </c>
       <c r="E968" s="9" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>0:43:48</t>
         </is>
       </c>
     </row>
     <row r="969">
       <c r="A969" s="4" t="inlineStr">
         <is>
-          <t>Broad Street Run</t>
+          <t>Boilermaker Road Race</t>
         </is>
       </c>
       <c r="B969" s="5" t="inlineStr">
@@ -24703,19 +24703,19 @@
       </c>
       <c r="D969" s="5" t="inlineStr">
         <is>
-          <t>0:46:13</t>
+          <t>0:42:44</t>
         </is>
       </c>
       <c r="E969" s="5" t="inlineStr">
         <is>
-          <t>0:54:01</t>
+          <t>N/A</t>
         </is>
       </c>
     </row>
     <row r="970">
       <c r="A970" s="8" t="inlineStr">
         <is>
-          <t>City2Surf</t>
+          <t>Broad Street Run</t>
         </is>
       </c>
       <c r="B970" s="9" t="inlineStr">
@@ -24724,16 +24724,16 @@
         </is>
       </c>
       <c r="C970" s="9" t="n">
-        <v>2024</v>
+        <v>2025</v>
       </c>
       <c r="D970" s="9" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>0:46:13</t>
         </is>
       </c>
       <c r="E970" s="9" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>0:54:01</t>
         </is>
       </c>
     </row>
@@ -24749,23 +24749,23 @@
         </is>
       </c>
       <c r="C971" s="5" t="n">
-        <v>2026</v>
+        <v>2024</v>
       </c>
       <c r="D971" s="5" t="inlineStr">
         <is>
-          <t>0:40:27</t>
+          <t>N/A</t>
         </is>
       </c>
       <c r="E971" s="5" t="inlineStr">
         <is>
-          <t>0:46:35</t>
+          <t>N/A</t>
         </is>
       </c>
     </row>
     <row r="972">
       <c r="A972" s="8" t="inlineStr">
         <is>
-          <t>Dam tot Damloop</t>
+          <t>City2Surf</t>
         </is>
       </c>
       <c r="B972" s="9" t="inlineStr">
@@ -24774,16 +24774,16 @@
         </is>
       </c>
       <c r="C972" s="9" t="n">
-        <v>2009</v>
+        <v>2026</v>
       </c>
       <c r="D972" s="9" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>0:40:27</t>
         </is>
       </c>
       <c r="E972" s="9" t="inlineStr">
         <is>
-          <t>0:50:39</t>
+          <t>0:46:35</t>
         </is>
       </c>
     </row>
@@ -24799,7 +24799,7 @@
         </is>
       </c>
       <c r="C973" s="5" t="n">
-        <v>2010</v>
+        <v>2009</v>
       </c>
       <c r="D973" s="5" t="inlineStr">
         <is>
@@ -24808,7 +24808,7 @@
       </c>
       <c r="E973" s="5" t="inlineStr">
         <is>
-          <t>0:51:30</t>
+          <t>0:50:39</t>
         </is>
       </c>
     </row>
@@ -24824,16 +24824,16 @@
         </is>
       </c>
       <c r="C974" s="9" t="n">
-        <v>2011</v>
+        <v>2010</v>
       </c>
       <c r="D974" s="9" t="inlineStr">
         <is>
-          <t>0:44:27</t>
+          <t>N/A</t>
         </is>
       </c>
       <c r="E974" s="9" t="inlineStr">
         <is>
-          <t>0:51:57</t>
+          <t>0:51:30</t>
         </is>
       </c>
     </row>
@@ -24849,16 +24849,16 @@
         </is>
       </c>
       <c r="C975" s="5" t="n">
-        <v>2012</v>
+        <v>2011</v>
       </c>
       <c r="D975" s="5" t="inlineStr">
         <is>
-          <t>0:44:48</t>
+          <t>0:44:27</t>
         </is>
       </c>
       <c r="E975" s="5" t="inlineStr">
         <is>
-          <t>0:51:42</t>
+          <t>0:51:57</t>
         </is>
       </c>
     </row>
@@ -24874,16 +24874,16 @@
         </is>
       </c>
       <c r="C976" s="9" t="n">
-        <v>2013</v>
+        <v>2012</v>
       </c>
       <c r="D976" s="9" t="inlineStr">
         <is>
-          <t>0:45:28</t>
+          <t>0:44:48</t>
         </is>
       </c>
       <c r="E976" s="9" t="inlineStr">
         <is>
-          <t>0:51:33</t>
+          <t>0:51:42</t>
         </is>
       </c>
     </row>
@@ -24899,16 +24899,16 @@
         </is>
       </c>
       <c r="C977" s="5" t="n">
-        <v>2014</v>
+        <v>2013</v>
       </c>
       <c r="D977" s="5" t="inlineStr">
         <is>
-          <t>0:45:45</t>
+          <t>0:45:28</t>
         </is>
       </c>
       <c r="E977" s="5" t="inlineStr">
         <is>
-          <t>0:53:09</t>
+          <t>0:51:33</t>
         </is>
       </c>
     </row>
@@ -24924,16 +24924,16 @@
         </is>
       </c>
       <c r="C978" s="9" t="n">
-        <v>2019</v>
+        <v>2014</v>
       </c>
       <c r="D978" s="9" t="inlineStr">
         <is>
-          <t>0:45:15</t>
+          <t>0:45:45</t>
         </is>
       </c>
       <c r="E978" s="9" t="inlineStr">
         <is>
-          <t>0:50:45</t>
+          <t>0:53:09</t>
         </is>
       </c>
     </row>
@@ -24949,16 +24949,16 @@
         </is>
       </c>
       <c r="C979" s="5" t="n">
-        <v>2022</v>
+        <v>2019</v>
       </c>
       <c r="D979" s="5" t="inlineStr">
         <is>
-          <t>0:49:00</t>
+          <t>0:45:15</t>
         </is>
       </c>
       <c r="E979" s="5" t="inlineStr">
         <is>
-          <t>0:55:44</t>
+          <t>0:50:45</t>
         </is>
       </c>
     </row>
@@ -24974,16 +24974,16 @@
         </is>
       </c>
       <c r="C980" s="9" t="n">
-        <v>2024</v>
+        <v>2022</v>
       </c>
       <c r="D980" s="9" t="inlineStr">
         <is>
-          <t>0:44:51</t>
+          <t>0:49:00</t>
         </is>
       </c>
       <c r="E980" s="9" t="inlineStr">
         <is>
-          <t>0:51:15</t>
+          <t>0:55:44</t>
         </is>
       </c>
     </row>
@@ -24999,23 +24999,23 @@
         </is>
       </c>
       <c r="C981" s="5" t="n">
-        <v>2025</v>
+        <v>2024</v>
       </c>
       <c r="D981" s="5" t="inlineStr">
         <is>
-          <t>0:46:07</t>
+          <t>0:44:51</t>
         </is>
       </c>
       <c r="E981" s="5" t="inlineStr">
         <is>
-          <t>0:50:51</t>
+          <t>0:51:15</t>
         </is>
       </c>
     </row>
     <row r="982">
       <c r="A982" s="8" t="inlineStr">
         <is>
-          <t>Falmouth Road Race</t>
+          <t>Dam tot Damloop</t>
         </is>
       </c>
       <c r="B982" s="9" t="inlineStr">
@@ -25028,19 +25028,19 @@
       </c>
       <c r="D982" s="9" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>0:46:07</t>
         </is>
       </c>
       <c r="E982" s="9" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>0:50:51</t>
         </is>
       </c>
     </row>
     <row r="983">
       <c r="A983" s="4" t="inlineStr">
         <is>
-          <t>Grand Prix Von Bern</t>
+          <t>Falmouth Road Race</t>
         </is>
       </c>
       <c r="B983" s="5" t="inlineStr">
@@ -25049,73 +25049,73 @@
         </is>
       </c>
       <c r="C983" s="5" t="n">
-        <v>2026</v>
+        <v>2025</v>
       </c>
       <c r="D983" s="5" t="inlineStr">
         <is>
-          <t>0:46:58</t>
+          <t>N/A</t>
         </is>
       </c>
       <c r="E983" s="5" t="inlineStr">
         <is>
-          <t>0:55:50</t>
+          <t>N/A</t>
         </is>
       </c>
     </row>
     <row r="984">
       <c r="A984" s="8" t="inlineStr">
         <is>
-          <t>Great Scottish Run</t>
+          <t>Grand Prix Von Bern</t>
         </is>
       </c>
       <c r="B984" s="9" t="inlineStr">
         <is>
-          <t>SEMI</t>
+          <t>AUTRE</t>
         </is>
       </c>
       <c r="C984" s="9" t="n">
-        <v>2025</v>
+        <v>2026</v>
       </c>
       <c r="D984" s="9" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>0:46:58</t>
         </is>
       </c>
       <c r="E984" s="9" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>0:55:50</t>
         </is>
       </c>
     </row>
     <row r="985">
       <c r="A985" s="4" t="inlineStr">
         <is>
-          <t>Harmonie Mutuelle 20km de Paris</t>
+          <t>Great Scottish Run</t>
         </is>
       </c>
       <c r="B985" s="5" t="inlineStr">
         <is>
-          <t>AUTRE</t>
+          <t>SEMI</t>
         </is>
       </c>
       <c r="C985" s="5" t="n">
-        <v>2026</v>
+        <v>2025</v>
       </c>
       <c r="D985" s="5" t="inlineStr">
         <is>
-          <t>00:57:11</t>
+          <t>N/A</t>
         </is>
       </c>
       <c r="E985" s="5" t="inlineStr">
         <is>
-          <t>01:04:35</t>
+          <t>N/A</t>
         </is>
       </c>
     </row>
     <row r="986">
       <c r="A986" s="8" t="inlineStr">
         <is>
-          <t>Lilac Bloomsday Run</t>
+          <t>Harmonie Mutuelle 20km de Paris</t>
         </is>
       </c>
       <c r="B986" s="9" t="inlineStr">
@@ -25124,23 +25124,23 @@
         </is>
       </c>
       <c r="C986" s="9" t="n">
-        <v>2025</v>
+        <v>2026</v>
       </c>
       <c r="D986" s="9" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>00:57:11</t>
         </is>
       </c>
       <c r="E986" s="9" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>01:04:35</t>
         </is>
       </c>
     </row>
     <row r="987">
       <c r="A987" s="4" t="inlineStr">
         <is>
-          <t>Manchester Road Race</t>
+          <t>Lilac Bloomsday Run</t>
         </is>
       </c>
       <c r="B987" s="5" t="inlineStr">
@@ -25149,7 +25149,7 @@
         </is>
       </c>
       <c r="C987" s="5" t="n">
-        <v>2024</v>
+        <v>2025</v>
       </c>
       <c r="D987" s="5" t="inlineStr">
         <is>
@@ -25165,30 +25165,55 @@
     <row r="988">
       <c r="A988" s="8" t="inlineStr">
         <is>
+          <t>Manchester Road Race</t>
+        </is>
+      </c>
+      <c r="B988" s="9" t="inlineStr">
+        <is>
+          <t>AUTRE</t>
+        </is>
+      </c>
+      <c r="C988" s="9" t="n">
+        <v>2024</v>
+      </c>
+      <c r="D988" s="9" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="E988" s="9" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+    </row>
+    <row r="989">
+      <c r="A989" s="4" t="inlineStr">
+        <is>
           <t>Paris-Versailles - La grande classique</t>
         </is>
       </c>
-      <c r="B988" s="9" t="inlineStr">
+      <c r="B989" s="5" t="inlineStr">
         <is>
           <t>AUTRE</t>
         </is>
       </c>
-      <c r="C988" s="9" t="n">
+      <c r="C989" s="5" t="n">
         <v>2026</v>
       </c>
-      <c r="D988" s="9" t="inlineStr">
+      <c r="D989" s="5" t="inlineStr">
         <is>
           <t>00:49:05</t>
         </is>
       </c>
-      <c r="E988" s="9" t="inlineStr">
+      <c r="E989" s="5" t="inlineStr">
         <is>
           <t>00:55:58</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:E988"/>
+  <autoFilter ref="A1:E989"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>